<commit_message>
Update trade value sheets
</commit_message>
<xml_diff>
--- a/TradeValueSheets/TradeValues_AllCombinations.xlsx
+++ b/TradeValueSheets/TradeValues_AllCombinations.xlsx
@@ -748,7 +748,7 @@
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
@@ -1134,13 +1134,13 @@
       <c r="A28" s="7" t="n">
         <v>34</v>
       </c>
-      <c r="B28" s="8" t="n"/>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>D'Andre Swift</t>
+        </is>
+      </c>
       <c r="C28" s="8" t="n"/>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>DeVonta Smith</t>
-        </is>
-      </c>
+      <c r="D28" s="8" t="n"/>
       <c r="E28" s="8" t="n"/>
       <c r="F28" s="8" t="n"/>
       <c r="G28" s="8" t="n"/>
@@ -1184,43 +1184,43 @@
       </c>
       <c r="B31" s="8" t="n"/>
       <c r="C31" s="8" t="n"/>
-      <c r="D31" s="8" t="n"/>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>DeVonta Smith</t>
+        </is>
+      </c>
       <c r="E31" s="8" t="n"/>
       <c r="F31" s="8" t="n"/>
       <c r="G31" s="8" t="n"/>
-      <c r="H31" s="8" t="inlineStr">
-        <is>
-          <t>Josh Allen</t>
-        </is>
-      </c>
+      <c r="H31" s="8" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B32" s="8" t="n"/>
       <c r="C32" s="8" t="n"/>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>A.J. Brown</t>
-        </is>
-      </c>
+      <c r="D32" s="8" t="n"/>
       <c r="E32" s="8" t="n"/>
       <c r="F32" s="8" t="n"/>
       <c r="G32" s="8" t="n"/>
-      <c r="H32" s="8" t="n"/>
+      <c r="H32" s="8" t="inlineStr">
+        <is>
+          <t>Josh Allen</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n">
-        <v>27</v>
-      </c>
-      <c r="B33" s="8" t="inlineStr">
-        <is>
-          <t>D'Andre Swift</t>
-        </is>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="B33" s="8" t="n"/>
       <c r="C33" s="8" t="n"/>
-      <c r="D33" s="8" t="n"/>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>A.J. Brown</t>
+        </is>
+      </c>
       <c r="E33" s="8" t="n"/>
       <c r="F33" s="8" t="n"/>
       <c r="G33" s="8" t="n"/>
@@ -1374,13 +1374,13 @@
       <c r="A43" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="B43" s="8" t="inlineStr">
-        <is>
-          <t>Cam Skattebo</t>
-        </is>
-      </c>
+      <c r="B43" s="8" t="n"/>
       <c r="C43" s="8" t="n"/>
-      <c r="D43" s="8" t="n"/>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Rashee Rice</t>
+        </is>
+      </c>
       <c r="E43" s="8" t="n"/>
       <c r="F43" s="8" t="n"/>
       <c r="G43" s="8" t="n"/>
@@ -1388,15 +1388,15 @@
     </row>
     <row r="44">
       <c r="A44" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="B44" s="8" t="n"/>
+        <v>19</v>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>Jeremiyah Love</t>
+        </is>
+      </c>
       <c r="C44" s="8" t="n"/>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Rashee Rice</t>
-        </is>
-      </c>
+      <c r="D44" s="8" t="n"/>
       <c r="E44" s="8" t="n"/>
       <c r="F44" s="8" t="n"/>
       <c r="G44" s="8" t="n"/>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>Jeremiyah Love</t>
+          <t>Cam Skattebo</t>
         </is>
       </c>
       <c r="C45" s="8" t="n"/>
@@ -1500,11 +1500,11 @@
     </row>
     <row r="51">
       <c r="A51" s="7" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>Quinshon Judkins</t>
+          <t>Chuba Hubbard</t>
         </is>
       </c>
       <c r="C51" s="8" t="n"/>
@@ -1516,11 +1516,11 @@
     </row>
     <row r="52">
       <c r="A52" s="7" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>Chuba Hubbard</t>
+          <t>Quinshon Judkins</t>
         </is>
       </c>
       <c r="C52" s="8" t="n"/>
@@ -2528,7 +2528,7 @@
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
@@ -2882,13 +2882,13 @@
       <c r="A26" s="7" t="n">
         <v>34</v>
       </c>
-      <c r="B26" s="8" t="n"/>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>D'Andre Swift</t>
+        </is>
+      </c>
       <c r="C26" s="8" t="n"/>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>Nico Collins</t>
-        </is>
-      </c>
+      <c r="D26" s="8" t="n"/>
       <c r="E26" s="8" t="n"/>
       <c r="F26" s="8" t="n"/>
       <c r="G26" s="8" t="n"/>
@@ -2896,15 +2896,15 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="n">
-        <v>33</v>
-      </c>
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>Omarion Hampton</t>
-        </is>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="B27" s="8" t="n"/>
       <c r="C27" s="8" t="n"/>
-      <c r="D27" s="8" t="n"/>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Nico Collins</t>
+        </is>
+      </c>
       <c r="E27" s="8" t="n"/>
       <c r="F27" s="8" t="n"/>
       <c r="G27" s="8" t="n"/>
@@ -2912,15 +2912,15 @@
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
-        <v>32</v>
-      </c>
-      <c r="B28" s="8" t="n"/>
+        <v>33</v>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Omarion Hampton</t>
+        </is>
+      </c>
       <c r="C28" s="8" t="n"/>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>Drake London</t>
-        </is>
-      </c>
+      <c r="D28" s="8" t="n"/>
       <c r="E28" s="8" t="n"/>
       <c r="F28" s="8" t="n"/>
       <c r="G28" s="8" t="n"/>
@@ -2934,7 +2934,7 @@
       <c r="C29" s="8" t="n"/>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>Garrett Wilson</t>
+          <t>Drake London</t>
         </is>
       </c>
       <c r="E29" s="8" t="n"/>
@@ -2950,7 +2950,7 @@
       <c r="C30" s="8" t="n"/>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>George Pickens</t>
+          <t>Garrett Wilson</t>
         </is>
       </c>
       <c r="E30" s="8" t="n"/>
@@ -2960,15 +2960,15 @@
     </row>
     <row r="31">
       <c r="A31" s="7" t="n">
-        <v>31</v>
-      </c>
-      <c r="B31" s="8" t="inlineStr">
-        <is>
-          <t>Kyren Williams</t>
-        </is>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="B31" s="8" t="n"/>
       <c r="C31" s="8" t="n"/>
-      <c r="D31" s="8" t="n"/>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>George Pickens</t>
+        </is>
+      </c>
       <c r="E31" s="8" t="n"/>
       <c r="F31" s="8" t="n"/>
       <c r="G31" s="8" t="n"/>
@@ -2976,15 +2976,15 @@
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="B32" s="8" t="n"/>
+        <v>31</v>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Kyren Williams</t>
+        </is>
+      </c>
       <c r="C32" s="8" t="n"/>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>DeVonta Smith</t>
-        </is>
-      </c>
+      <c r="D32" s="8" t="n"/>
       <c r="E32" s="8" t="n"/>
       <c r="F32" s="8" t="n"/>
       <c r="G32" s="8" t="n"/>
@@ -2998,7 +2998,7 @@
       <c r="C33" s="8" t="n"/>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>A.J. Brown</t>
+          <t>DeVonta Smith</t>
         </is>
       </c>
       <c r="E33" s="8" t="n"/>
@@ -3008,15 +3008,15 @@
     </row>
     <row r="34">
       <c r="A34" s="7" t="n">
-        <v>29</v>
-      </c>
-      <c r="B34" s="8" t="inlineStr">
-        <is>
-          <t>D'Andre Swift</t>
-        </is>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="B34" s="8" t="n"/>
       <c r="C34" s="8" t="n"/>
-      <c r="D34" s="8" t="n"/>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>A.J. Brown</t>
+        </is>
+      </c>
       <c r="E34" s="8" t="n"/>
       <c r="F34" s="8" t="n"/>
       <c r="G34" s="8" t="n"/>
@@ -3122,13 +3122,13 @@
       <c r="A41" s="7" t="n">
         <v>23</v>
       </c>
-      <c r="B41" s="8" t="inlineStr">
-        <is>
-          <t>Quinshon Judkins</t>
-        </is>
-      </c>
+      <c r="B41" s="8" t="n"/>
       <c r="C41" s="8" t="n"/>
-      <c r="D41" s="8" t="n"/>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Parker Washington</t>
+        </is>
+      </c>
       <c r="E41" s="8" t="n"/>
       <c r="F41" s="8" t="n"/>
       <c r="G41" s="8" t="n"/>
@@ -3136,15 +3136,15 @@
     </row>
     <row r="42">
       <c r="A42" s="7" t="n">
-        <v>23</v>
-      </c>
-      <c r="B42" s="8" t="n"/>
+        <v>22</v>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>Chuba Hubbard</t>
+        </is>
+      </c>
       <c r="C42" s="8" t="n"/>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>Parker Washington</t>
-        </is>
-      </c>
+      <c r="D42" s="8" t="n"/>
       <c r="E42" s="8" t="n"/>
       <c r="F42" s="8" t="n"/>
       <c r="G42" s="8" t="n"/>
@@ -3154,13 +3154,13 @@
       <c r="A43" s="7" t="n">
         <v>22</v>
       </c>
-      <c r="B43" s="8" t="inlineStr">
-        <is>
-          <t>Cam Skattebo</t>
-        </is>
-      </c>
+      <c r="B43" s="8" t="n"/>
       <c r="C43" s="8" t="n"/>
-      <c r="D43" s="8" t="n"/>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Ladd McConkey</t>
+        </is>
+      </c>
       <c r="E43" s="8" t="n"/>
       <c r="F43" s="8" t="n"/>
       <c r="G43" s="8" t="n"/>
@@ -3168,11 +3168,11 @@
     </row>
     <row r="44">
       <c r="A44" s="7" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>Chuba Hubbard</t>
+          <t>Jeremiyah Love</t>
         </is>
       </c>
       <c r="C44" s="8" t="n"/>
@@ -3184,15 +3184,15 @@
     </row>
     <row r="45">
       <c r="A45" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="B45" s="8" t="n"/>
+        <v>21</v>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>Cam Skattebo</t>
+        </is>
+      </c>
       <c r="C45" s="8" t="n"/>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>Ladd McConkey</t>
-        </is>
-      </c>
+      <c r="D45" s="8" t="n"/>
       <c r="E45" s="8" t="n"/>
       <c r="F45" s="8" t="n"/>
       <c r="G45" s="8" t="n"/>
@@ -3204,7 +3204,7 @@
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>Jeremiyah Love</t>
+          <t>Quinshon Judkins</t>
         </is>
       </c>
       <c r="C46" s="8" t="n"/>
@@ -4308,7 +4308,7 @@
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
@@ -4662,13 +4662,13 @@
       <c r="A26" s="7" t="n">
         <v>33</v>
       </c>
-      <c r="B26" s="8" t="n"/>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>D'Andre Swift</t>
+        </is>
+      </c>
       <c r="C26" s="8" t="n"/>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>Nico Collins</t>
-        </is>
-      </c>
+      <c r="D26" s="8" t="n"/>
       <c r="E26" s="8" t="n"/>
       <c r="F26" s="8" t="n"/>
       <c r="G26" s="8" t="n"/>
@@ -4676,15 +4676,15 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="n">
-        <v>32</v>
-      </c>
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>Omarion Hampton</t>
-        </is>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="B27" s="8" t="n"/>
       <c r="C27" s="8" t="n"/>
-      <c r="D27" s="8" t="n"/>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Nico Collins</t>
+        </is>
+      </c>
       <c r="E27" s="8" t="n"/>
       <c r="F27" s="8" t="n"/>
       <c r="G27" s="8" t="n"/>
@@ -4694,13 +4694,13 @@
       <c r="A28" s="7" t="n">
         <v>32</v>
       </c>
-      <c r="B28" s="8" t="n"/>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Omarion Hampton</t>
+        </is>
+      </c>
       <c r="C28" s="8" t="n"/>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>George Pickens</t>
-        </is>
-      </c>
+      <c r="D28" s="8" t="n"/>
       <c r="E28" s="8" t="n"/>
       <c r="F28" s="8" t="n"/>
       <c r="G28" s="8" t="n"/>
@@ -4708,13 +4708,13 @@
     </row>
     <row r="29">
       <c r="A29" s="7" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B29" s="8" t="n"/>
       <c r="C29" s="8" t="n"/>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>Drake London</t>
+          <t>George Pickens</t>
         </is>
       </c>
       <c r="E29" s="8" t="n"/>
@@ -4730,7 +4730,7 @@
       <c r="C30" s="8" t="n"/>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>Garrett Wilson</t>
+          <t>Drake London</t>
         </is>
       </c>
       <c r="E30" s="8" t="n"/>
@@ -4740,15 +4740,15 @@
     </row>
     <row r="31">
       <c r="A31" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="8" t="inlineStr">
-        <is>
-          <t>Kyren Williams</t>
-        </is>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="B31" s="8" t="n"/>
       <c r="C31" s="8" t="n"/>
-      <c r="D31" s="8" t="n"/>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Garrett Wilson</t>
+        </is>
+      </c>
       <c r="E31" s="8" t="n"/>
       <c r="F31" s="8" t="n"/>
       <c r="G31" s="8" t="n"/>
@@ -4756,15 +4756,15 @@
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
-        <v>29</v>
-      </c>
-      <c r="B32" s="8" t="n"/>
+        <v>30</v>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Kyren Williams</t>
+        </is>
+      </c>
       <c r="C32" s="8" t="n"/>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>DeVonta Smith</t>
-        </is>
-      </c>
+      <c r="D32" s="8" t="n"/>
       <c r="E32" s="8" t="n"/>
       <c r="F32" s="8" t="n"/>
       <c r="G32" s="8" t="n"/>
@@ -4778,7 +4778,7 @@
       <c r="C33" s="8" t="n"/>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>A.J. Brown</t>
+          <t>DeVonta Smith</t>
         </is>
       </c>
       <c r="E33" s="8" t="n"/>
@@ -4792,31 +4792,31 @@
       </c>
       <c r="B34" s="8" t="n"/>
       <c r="C34" s="8" t="n"/>
-      <c r="D34" s="8" t="n"/>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>A.J. Brown</t>
+        </is>
+      </c>
       <c r="E34" s="8" t="n"/>
       <c r="F34" s="8" t="n"/>
       <c r="G34" s="8" t="n"/>
-      <c r="H34" s="8" t="inlineStr">
-        <is>
-          <t>Lamar Jackson</t>
-        </is>
-      </c>
+      <c r="H34" s="8" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n">
-        <v>27</v>
-      </c>
-      <c r="B35" s="8" t="inlineStr">
-        <is>
-          <t>D'Andre Swift</t>
-        </is>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="B35" s="8" t="n"/>
       <c r="C35" s="8" t="n"/>
       <c r="D35" s="8" t="n"/>
       <c r="E35" s="8" t="n"/>
       <c r="F35" s="8" t="n"/>
       <c r="G35" s="8" t="n"/>
-      <c r="H35" s="8" t="n"/>
+      <c r="H35" s="8" t="inlineStr">
+        <is>
+          <t>Lamar Jackson</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n">
@@ -4916,11 +4916,11 @@
     </row>
     <row r="42">
       <c r="A42" s="7" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>Quinshon Judkins</t>
+          <t>Chuba Hubbard</t>
         </is>
       </c>
       <c r="C42" s="8" t="n"/>
@@ -4934,13 +4934,13 @@
       <c r="A43" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="B43" s="8" t="inlineStr">
-        <is>
-          <t>Cam Skattebo</t>
-        </is>
-      </c>
+      <c r="B43" s="8" t="n"/>
       <c r="C43" s="8" t="n"/>
-      <c r="D43" s="8" t="n"/>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Ladd McConkey</t>
+        </is>
+      </c>
       <c r="E43" s="8" t="n"/>
       <c r="F43" s="8" t="n"/>
       <c r="G43" s="8" t="n"/>
@@ -4948,11 +4948,11 @@
     </row>
     <row r="44">
       <c r="A44" s="7" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>Chuba Hubbard</t>
+          <t>Jeremiyah Love</t>
         </is>
       </c>
       <c r="C44" s="8" t="n"/>
@@ -4964,15 +4964,15 @@
     </row>
     <row r="45">
       <c r="A45" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="B45" s="8" t="n"/>
+        <v>19</v>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>Cam Skattebo</t>
+        </is>
+      </c>
       <c r="C45" s="8" t="n"/>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>Ladd McConkey</t>
-        </is>
-      </c>
+      <c r="D45" s="8" t="n"/>
       <c r="E45" s="8" t="n"/>
       <c r="F45" s="8" t="n"/>
       <c r="G45" s="8" t="n"/>
@@ -4984,7 +4984,7 @@
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>Jeremiyah Love</t>
+          <t>Quinshon Judkins</t>
         </is>
       </c>
       <c r="C46" s="8" t="n"/>
@@ -6088,7 +6088,7 @@
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
@@ -6442,13 +6442,13 @@
       <c r="A26" s="7" t="n">
         <v>32</v>
       </c>
-      <c r="B26" s="8" t="n"/>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>D'Andre Swift</t>
+        </is>
+      </c>
       <c r="C26" s="8" t="n"/>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>Nico Collins</t>
-        </is>
-      </c>
+      <c r="D26" s="8" t="n"/>
       <c r="E26" s="8" t="n"/>
       <c r="F26" s="8" t="n"/>
       <c r="G26" s="8" t="n"/>
@@ -6456,15 +6456,15 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="n">
-        <v>31</v>
-      </c>
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>Omarion Hampton</t>
-        </is>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="B27" s="8" t="n"/>
       <c r="C27" s="8" t="n"/>
-      <c r="D27" s="8" t="n"/>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Nico Collins</t>
+        </is>
+      </c>
       <c r="E27" s="8" t="n"/>
       <c r="F27" s="8" t="n"/>
       <c r="G27" s="8" t="n"/>
@@ -6472,15 +6472,15 @@
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="B28" s="8" t="n"/>
+        <v>31</v>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Omarion Hampton</t>
+        </is>
+      </c>
       <c r="C28" s="8" t="n"/>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>Drake London</t>
-        </is>
-      </c>
+      <c r="D28" s="8" t="n"/>
       <c r="E28" s="8" t="n"/>
       <c r="F28" s="8" t="n"/>
       <c r="G28" s="8" t="n"/>
@@ -6494,7 +6494,7 @@
       <c r="C29" s="8" t="n"/>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>Garrett Wilson</t>
+          <t>Drake London</t>
         </is>
       </c>
       <c r="E29" s="8" t="n"/>
@@ -6510,7 +6510,7 @@
       <c r="C30" s="8" t="n"/>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>George Pickens</t>
+          <t>Garrett Wilson</t>
         </is>
       </c>
       <c r="E30" s="8" t="n"/>
@@ -6520,15 +6520,15 @@
     </row>
     <row r="31">
       <c r="A31" s="7" t="n">
-        <v>28</v>
-      </c>
-      <c r="B31" s="8" t="inlineStr">
-        <is>
-          <t>Kyren Williams</t>
-        </is>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="B31" s="8" t="n"/>
       <c r="C31" s="8" t="n"/>
-      <c r="D31" s="8" t="n"/>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>George Pickens</t>
+        </is>
+      </c>
       <c r="E31" s="8" t="n"/>
       <c r="F31" s="8" t="n"/>
       <c r="G31" s="8" t="n"/>
@@ -6536,15 +6536,15 @@
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
-        <v>27</v>
-      </c>
-      <c r="B32" s="8" t="n"/>
+        <v>28</v>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Kyren Williams</t>
+        </is>
+      </c>
       <c r="C32" s="8" t="n"/>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>DeVonta Smith</t>
-        </is>
-      </c>
+      <c r="D32" s="8" t="n"/>
       <c r="E32" s="8" t="n"/>
       <c r="F32" s="8" t="n"/>
       <c r="G32" s="8" t="n"/>
@@ -6572,31 +6572,31 @@
       </c>
       <c r="B34" s="8" t="n"/>
       <c r="C34" s="8" t="n"/>
-      <c r="D34" s="8" t="n"/>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>DeVonta Smith</t>
+        </is>
+      </c>
       <c r="E34" s="8" t="n"/>
       <c r="F34" s="8" t="n"/>
       <c r="G34" s="8" t="n"/>
-      <c r="H34" s="8" t="inlineStr">
-        <is>
-          <t>Lamar Jackson</t>
-        </is>
-      </c>
+      <c r="H34" s="8" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n">
-        <v>25</v>
-      </c>
-      <c r="B35" s="8" t="inlineStr">
-        <is>
-          <t>D'Andre Swift</t>
-        </is>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="B35" s="8" t="n"/>
       <c r="C35" s="8" t="n"/>
       <c r="D35" s="8" t="n"/>
       <c r="E35" s="8" t="n"/>
       <c r="F35" s="8" t="n"/>
       <c r="G35" s="8" t="n"/>
-      <c r="H35" s="8" t="n"/>
+      <c r="H35" s="8" t="inlineStr">
+        <is>
+          <t>Lamar Jackson</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n">
@@ -6682,13 +6682,13 @@
       <c r="A41" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="B41" s="8" t="inlineStr">
-        <is>
-          <t>Quinshon Judkins</t>
-        </is>
-      </c>
+      <c r="B41" s="8" t="n"/>
       <c r="C41" s="8" t="n"/>
-      <c r="D41" s="8" t="n"/>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Parker Washington</t>
+        </is>
+      </c>
       <c r="E41" s="8" t="n"/>
       <c r="F41" s="8" t="n"/>
       <c r="G41" s="8" t="n"/>
@@ -6696,15 +6696,15 @@
     </row>
     <row r="42">
       <c r="A42" s="7" t="n">
-        <v>19</v>
-      </c>
-      <c r="B42" s="8" t="n"/>
+        <v>18</v>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>Chuba Hubbard</t>
+        </is>
+      </c>
       <c r="C42" s="8" t="n"/>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>Parker Washington</t>
-        </is>
-      </c>
+      <c r="D42" s="8" t="n"/>
       <c r="E42" s="8" t="n"/>
       <c r="F42" s="8" t="n"/>
       <c r="G42" s="8" t="n"/>
@@ -6714,13 +6714,13 @@
       <c r="A43" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="B43" s="8" t="inlineStr">
-        <is>
-          <t>Cam Skattebo</t>
-        </is>
-      </c>
+      <c r="B43" s="8" t="n"/>
       <c r="C43" s="8" t="n"/>
-      <c r="D43" s="8" t="n"/>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Ladd McConkey</t>
+        </is>
+      </c>
       <c r="E43" s="8" t="n"/>
       <c r="F43" s="8" t="n"/>
       <c r="G43" s="8" t="n"/>
@@ -6728,11 +6728,11 @@
     </row>
     <row r="44">
       <c r="A44" s="7" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>Chuba Hubbard</t>
+          <t>Jeremiyah Love</t>
         </is>
       </c>
       <c r="C44" s="8" t="n"/>
@@ -6744,15 +6744,15 @@
     </row>
     <row r="45">
       <c r="A45" s="7" t="n">
-        <v>18</v>
-      </c>
-      <c r="B45" s="8" t="n"/>
+        <v>17</v>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>Cam Skattebo</t>
+        </is>
+      </c>
       <c r="C45" s="8" t="n"/>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>Ladd McConkey</t>
-        </is>
-      </c>
+      <c r="D45" s="8" t="n"/>
       <c r="E45" s="8" t="n"/>
       <c r="F45" s="8" t="n"/>
       <c r="G45" s="8" t="n"/>
@@ -6764,7 +6764,7 @@
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>Jeremiyah Love</t>
+          <t>Quinshon Judkins</t>
         </is>
       </c>
       <c r="C46" s="8" t="n"/>
@@ -8238,13 +8238,13 @@
       <c r="A27" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="B27" s="8" t="n"/>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>D'Andre Swift</t>
+        </is>
+      </c>
       <c r="C27" s="8" t="n"/>
-      <c r="D27" s="8" t="inlineStr">
-        <is>
-          <t>Drake London</t>
-        </is>
-      </c>
+      <c r="D27" s="8" t="n"/>
       <c r="E27" s="8" t="n"/>
       <c r="F27" s="8" t="n"/>
       <c r="G27" s="8" t="n"/>
@@ -8258,7 +8258,7 @@
       <c r="C28" s="8" t="n"/>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>Garrett Wilson</t>
+          <t>Drake London</t>
         </is>
       </c>
       <c r="E28" s="8" t="n"/>
@@ -8268,15 +8268,15 @@
     </row>
     <row r="29">
       <c r="A29" s="7" t="n">
-        <v>34</v>
-      </c>
-      <c r="B29" s="8" t="inlineStr">
-        <is>
-          <t>Omarion Hampton</t>
-        </is>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="B29" s="8" t="n"/>
       <c r="C29" s="8" t="n"/>
-      <c r="D29" s="8" t="n"/>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Garrett Wilson</t>
+        </is>
+      </c>
       <c r="E29" s="8" t="n"/>
       <c r="F29" s="8" t="n"/>
       <c r="G29" s="8" t="n"/>
@@ -8286,13 +8286,13 @@
       <c r="A30" s="7" t="n">
         <v>34</v>
       </c>
-      <c r="B30" s="8" t="n"/>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>Omarion Hampton</t>
+        </is>
+      </c>
       <c r="C30" s="8" t="n"/>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>George Pickens</t>
-        </is>
-      </c>
+      <c r="D30" s="8" t="n"/>
       <c r="E30" s="8" t="n"/>
       <c r="F30" s="8" t="n"/>
       <c r="G30" s="8" t="n"/>
@@ -8300,13 +8300,13 @@
     </row>
     <row r="31">
       <c r="A31" s="7" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B31" s="8" t="n"/>
       <c r="C31" s="8" t="n"/>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>DeVonta Smith</t>
+          <t>George Pickens</t>
         </is>
       </c>
       <c r="E31" s="8" t="n"/>
@@ -8316,13 +8316,13 @@
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B32" s="8" t="n"/>
       <c r="C32" s="8" t="n"/>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>A.J. Brown</t>
+          <t>DeVonta Smith</t>
         </is>
       </c>
       <c r="E32" s="8" t="n"/>
@@ -8332,15 +8332,15 @@
     </row>
     <row r="33">
       <c r="A33" s="7" t="n">
-        <v>29</v>
-      </c>
-      <c r="B33" s="8" t="inlineStr">
-        <is>
-          <t>D'Andre Swift</t>
-        </is>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="B33" s="8" t="n"/>
       <c r="C33" s="8" t="n"/>
-      <c r="D33" s="8" t="n"/>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>A.J. Brown</t>
+        </is>
+      </c>
       <c r="E33" s="8" t="n"/>
       <c r="F33" s="8" t="n"/>
       <c r="G33" s="8" t="n"/>
@@ -8478,13 +8478,13 @@
       <c r="A42" s="7" t="n">
         <v>23</v>
       </c>
-      <c r="B42" s="8" t="inlineStr">
-        <is>
-          <t>Cam Skattebo</t>
-        </is>
-      </c>
+      <c r="B42" s="8" t="n"/>
       <c r="C42" s="8" t="n"/>
-      <c r="D42" s="8" t="n"/>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Malik Nabers</t>
+        </is>
+      </c>
       <c r="E42" s="8" t="n"/>
       <c r="F42" s="8" t="n"/>
       <c r="G42" s="8" t="n"/>
@@ -8498,7 +8498,7 @@
       <c r="C43" s="8" t="n"/>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>Malik Nabers</t>
+          <t>Christian Watson</t>
         </is>
       </c>
       <c r="E43" s="8" t="n"/>
@@ -8508,15 +8508,15 @@
     </row>
     <row r="44">
       <c r="A44" s="7" t="n">
-        <v>23</v>
-      </c>
-      <c r="B44" s="8" t="n"/>
+        <v>22</v>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>Jeremiyah Love</t>
+        </is>
+      </c>
       <c r="C44" s="8" t="n"/>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Christian Watson</t>
-        </is>
-      </c>
+      <c r="D44" s="8" t="n"/>
       <c r="E44" s="8" t="n"/>
       <c r="F44" s="8" t="n"/>
       <c r="G44" s="8" t="n"/>
@@ -8528,7 +8528,7 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>Jeremiyah Love</t>
+          <t>Cam Skattebo</t>
         </is>
       </c>
       <c r="C45" s="8" t="n"/>
@@ -8574,13 +8574,13 @@
       <c r="A48" s="7" t="n">
         <v>21</v>
       </c>
-      <c r="B48" s="8" t="inlineStr">
-        <is>
-          <t>Quinshon Judkins</t>
-        </is>
-      </c>
+      <c r="B48" s="8" t="n"/>
       <c r="C48" s="8" t="n"/>
-      <c r="D48" s="8" t="n"/>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Rashee Rice</t>
+        </is>
+      </c>
       <c r="E48" s="8" t="n"/>
       <c r="F48" s="8" t="n"/>
       <c r="G48" s="8" t="n"/>
@@ -8588,15 +8588,15 @@
     </row>
     <row r="49">
       <c r="A49" s="7" t="n">
-        <v>21</v>
-      </c>
-      <c r="B49" s="8" t="n"/>
+        <v>20</v>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>Bucky Irving</t>
+        </is>
+      </c>
       <c r="C49" s="8" t="n"/>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Rashee Rice</t>
-        </is>
-      </c>
+      <c r="D49" s="8" t="n"/>
       <c r="E49" s="8" t="n"/>
       <c r="F49" s="8" t="n"/>
       <c r="G49" s="8" t="n"/>
@@ -8608,7 +8608,7 @@
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>Bucky Irving</t>
+          <t>Chuba Hubbard</t>
         </is>
       </c>
       <c r="C50" s="8" t="n"/>
@@ -8620,11 +8620,11 @@
     </row>
     <row r="51">
       <c r="A51" s="7" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>Chuba Hubbard</t>
+          <t>Quinshon Judkins</t>
         </is>
       </c>
       <c r="C51" s="8" t="n"/>
@@ -9648,7 +9648,7 @@
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
@@ -10018,13 +10018,13 @@
       <c r="A27" s="7" t="n">
         <v>34</v>
       </c>
-      <c r="B27" s="8" t="n"/>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>D'Andre Swift</t>
+        </is>
+      </c>
       <c r="C27" s="8" t="n"/>
-      <c r="D27" s="8" t="inlineStr">
-        <is>
-          <t>Drake London</t>
-        </is>
-      </c>
+      <c r="D27" s="8" t="n"/>
       <c r="E27" s="8" t="n"/>
       <c r="F27" s="8" t="n"/>
       <c r="G27" s="8" t="n"/>
@@ -10038,7 +10038,7 @@
       <c r="C28" s="8" t="n"/>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>Garrett Wilson</t>
+          <t>Drake London</t>
         </is>
       </c>
       <c r="E28" s="8" t="n"/>
@@ -10048,15 +10048,15 @@
     </row>
     <row r="29">
       <c r="A29" s="7" t="n">
-        <v>33</v>
-      </c>
-      <c r="B29" s="8" t="inlineStr">
-        <is>
-          <t>Omarion Hampton</t>
-        </is>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="B29" s="8" t="n"/>
       <c r="C29" s="8" t="n"/>
-      <c r="D29" s="8" t="n"/>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Garrett Wilson</t>
+        </is>
+      </c>
       <c r="E29" s="8" t="n"/>
       <c r="F29" s="8" t="n"/>
       <c r="G29" s="8" t="n"/>
@@ -10066,13 +10066,13 @@
       <c r="A30" s="7" t="n">
         <v>33</v>
       </c>
-      <c r="B30" s="8" t="n"/>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>Omarion Hampton</t>
+        </is>
+      </c>
       <c r="C30" s="8" t="n"/>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>George Pickens</t>
-        </is>
-      </c>
+      <c r="D30" s="8" t="n"/>
       <c r="E30" s="8" t="n"/>
       <c r="F30" s="8" t="n"/>
       <c r="G30" s="8" t="n"/>
@@ -10080,13 +10080,13 @@
     </row>
     <row r="31">
       <c r="A31" s="7" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B31" s="8" t="n"/>
       <c r="C31" s="8" t="n"/>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>DeVonta Smith</t>
+          <t>George Pickens</t>
         </is>
       </c>
       <c r="E31" s="8" t="n"/>
@@ -10096,13 +10096,13 @@
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B32" s="8" t="n"/>
       <c r="C32" s="8" t="n"/>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>A.J. Brown</t>
+          <t>DeVonta Smith</t>
         </is>
       </c>
       <c r="E32" s="8" t="n"/>
@@ -10112,15 +10112,15 @@
     </row>
     <row r="33">
       <c r="A33" s="7" t="n">
-        <v>28</v>
-      </c>
-      <c r="B33" s="8" t="inlineStr">
-        <is>
-          <t>D'Andre Swift</t>
-        </is>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="B33" s="8" t="n"/>
       <c r="C33" s="8" t="n"/>
-      <c r="D33" s="8" t="n"/>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>A.J. Brown</t>
+        </is>
+      </c>
       <c r="E33" s="8" t="n"/>
       <c r="F33" s="8" t="n"/>
       <c r="G33" s="8" t="n"/>
@@ -10258,13 +10258,13 @@
       <c r="A42" s="7" t="n">
         <v>21</v>
       </c>
-      <c r="B42" s="8" t="inlineStr">
-        <is>
-          <t>Cam Skattebo</t>
-        </is>
-      </c>
+      <c r="B42" s="8" t="n"/>
       <c r="C42" s="8" t="n"/>
-      <c r="D42" s="8" t="n"/>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Malik Nabers</t>
+        </is>
+      </c>
       <c r="E42" s="8" t="n"/>
       <c r="F42" s="8" t="n"/>
       <c r="G42" s="8" t="n"/>
@@ -10278,7 +10278,7 @@
       <c r="C43" s="8" t="n"/>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>Malik Nabers</t>
+          <t>Christian Watson</t>
         </is>
       </c>
       <c r="E43" s="8" t="n"/>
@@ -10288,15 +10288,15 @@
     </row>
     <row r="44">
       <c r="A44" s="7" t="n">
-        <v>21</v>
-      </c>
-      <c r="B44" s="8" t="n"/>
+        <v>20</v>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>Jeremiyah Love</t>
+        </is>
+      </c>
       <c r="C44" s="8" t="n"/>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Christian Watson</t>
-        </is>
-      </c>
+      <c r="D44" s="8" t="n"/>
       <c r="E44" s="8" t="n"/>
       <c r="F44" s="8" t="n"/>
       <c r="G44" s="8" t="n"/>
@@ -10308,7 +10308,7 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>Jeremiyah Love</t>
+          <t>Cam Skattebo</t>
         </is>
       </c>
       <c r="C45" s="8" t="n"/>
@@ -10354,13 +10354,13 @@
       <c r="A48" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="B48" s="8" t="inlineStr">
-        <is>
-          <t>Quinshon Judkins</t>
-        </is>
-      </c>
+      <c r="B48" s="8" t="n"/>
       <c r="C48" s="8" t="n"/>
-      <c r="D48" s="8" t="n"/>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Rashee Rice</t>
+        </is>
+      </c>
       <c r="E48" s="8" t="n"/>
       <c r="F48" s="8" t="n"/>
       <c r="G48" s="8" t="n"/>
@@ -10368,15 +10368,15 @@
     </row>
     <row r="49">
       <c r="A49" s="7" t="n">
-        <v>19</v>
-      </c>
-      <c r="B49" s="8" t="n"/>
+        <v>18</v>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>Bucky Irving</t>
+        </is>
+      </c>
       <c r="C49" s="8" t="n"/>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Rashee Rice</t>
-        </is>
-      </c>
+      <c r="D49" s="8" t="n"/>
       <c r="E49" s="8" t="n"/>
       <c r="F49" s="8" t="n"/>
       <c r="G49" s="8" t="n"/>
@@ -10388,7 +10388,7 @@
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>Bucky Irving</t>
+          <t>Chuba Hubbard</t>
         </is>
       </c>
       <c r="C50" s="8" t="n"/>
@@ -10400,11 +10400,11 @@
     </row>
     <row r="51">
       <c r="A51" s="7" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>Chuba Hubbard</t>
+          <t>Quinshon Judkins</t>
         </is>
       </c>
       <c r="C51" s="8" t="n"/>
@@ -11428,7 +11428,7 @@
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
@@ -11798,13 +11798,13 @@
       <c r="A27" s="7" t="n">
         <v>33</v>
       </c>
-      <c r="B27" s="8" t="n"/>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>D'Andre Swift</t>
+        </is>
+      </c>
       <c r="C27" s="8" t="n"/>
-      <c r="D27" s="8" t="inlineStr">
-        <is>
-          <t>Drake London</t>
-        </is>
-      </c>
+      <c r="D27" s="8" t="n"/>
       <c r="E27" s="8" t="n"/>
       <c r="F27" s="8" t="n"/>
       <c r="G27" s="8" t="n"/>
@@ -11818,7 +11818,7 @@
       <c r="C28" s="8" t="n"/>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>Garrett Wilson</t>
+          <t>Drake London</t>
         </is>
       </c>
       <c r="E28" s="8" t="n"/>
@@ -11828,15 +11828,15 @@
     </row>
     <row r="29">
       <c r="A29" s="7" t="n">
-        <v>32</v>
-      </c>
-      <c r="B29" s="8" t="inlineStr">
-        <is>
-          <t>Omarion Hampton</t>
-        </is>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="B29" s="8" t="n"/>
       <c r="C29" s="8" t="n"/>
-      <c r="D29" s="8" t="n"/>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Garrett Wilson</t>
+        </is>
+      </c>
       <c r="E29" s="8" t="n"/>
       <c r="F29" s="8" t="n"/>
       <c r="G29" s="8" t="n"/>
@@ -11846,13 +11846,13 @@
       <c r="A30" s="7" t="n">
         <v>32</v>
       </c>
-      <c r="B30" s="8" t="n"/>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>Omarion Hampton</t>
+        </is>
+      </c>
       <c r="C30" s="8" t="n"/>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>George Pickens</t>
-        </is>
-      </c>
+      <c r="D30" s="8" t="n"/>
       <c r="E30" s="8" t="n"/>
       <c r="F30" s="8" t="n"/>
       <c r="G30" s="8" t="n"/>
@@ -11860,13 +11860,13 @@
     </row>
     <row r="31">
       <c r="A31" s="7" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B31" s="8" t="n"/>
       <c r="C31" s="8" t="n"/>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>DeVonta Smith</t>
+          <t>George Pickens</t>
         </is>
       </c>
       <c r="E31" s="8" t="n"/>
@@ -11876,13 +11876,13 @@
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B32" s="8" t="n"/>
       <c r="C32" s="8" t="n"/>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>A.J. Brown</t>
+          <t>DeVonta Smith</t>
         </is>
       </c>
       <c r="E32" s="8" t="n"/>
@@ -11892,15 +11892,15 @@
     </row>
     <row r="33">
       <c r="A33" s="7" t="n">
-        <v>26</v>
-      </c>
-      <c r="B33" s="8" t="inlineStr">
-        <is>
-          <t>D'Andre Swift</t>
-        </is>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="B33" s="8" t="n"/>
       <c r="C33" s="8" t="n"/>
-      <c r="D33" s="8" t="n"/>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>A.J. Brown</t>
+        </is>
+      </c>
       <c r="E33" s="8" t="n"/>
       <c r="F33" s="8" t="n"/>
       <c r="G33" s="8" t="n"/>
@@ -12038,13 +12038,13 @@
       <c r="A42" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="B42" s="8" t="inlineStr">
-        <is>
-          <t>Cam Skattebo</t>
-        </is>
-      </c>
+      <c r="B42" s="8" t="n"/>
       <c r="C42" s="8" t="n"/>
-      <c r="D42" s="8" t="n"/>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Malik Nabers</t>
+        </is>
+      </c>
       <c r="E42" s="8" t="n"/>
       <c r="F42" s="8" t="n"/>
       <c r="G42" s="8" t="n"/>
@@ -12058,7 +12058,7 @@
       <c r="C43" s="8" t="n"/>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>Malik Nabers</t>
+          <t>Christian Watson</t>
         </is>
       </c>
       <c r="E43" s="8" t="n"/>
@@ -12068,15 +12068,15 @@
     </row>
     <row r="44">
       <c r="A44" s="7" t="n">
-        <v>19</v>
-      </c>
-      <c r="B44" s="8" t="n"/>
+        <v>18</v>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>Jeremiyah Love</t>
+        </is>
+      </c>
       <c r="C44" s="8" t="n"/>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Christian Watson</t>
-        </is>
-      </c>
+      <c r="D44" s="8" t="n"/>
       <c r="E44" s="8" t="n"/>
       <c r="F44" s="8" t="n"/>
       <c r="G44" s="8" t="n"/>
@@ -12088,7 +12088,7 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>Jeremiyah Love</t>
+          <t>Cam Skattebo</t>
         </is>
       </c>
       <c r="C45" s="8" t="n"/>
@@ -12134,13 +12134,13 @@
       <c r="A48" s="7" t="n">
         <v>17</v>
       </c>
-      <c r="B48" s="8" t="inlineStr">
-        <is>
-          <t>Quinshon Judkins</t>
-        </is>
-      </c>
+      <c r="B48" s="8" t="n"/>
       <c r="C48" s="8" t="n"/>
-      <c r="D48" s="8" t="n"/>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Rashee Rice</t>
+        </is>
+      </c>
       <c r="E48" s="8" t="n"/>
       <c r="F48" s="8" t="n"/>
       <c r="G48" s="8" t="n"/>
@@ -12148,15 +12148,15 @@
     </row>
     <row r="49">
       <c r="A49" s="7" t="n">
-        <v>17</v>
-      </c>
-      <c r="B49" s="8" t="n"/>
+        <v>16</v>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>Bucky Irving</t>
+        </is>
+      </c>
       <c r="C49" s="8" t="n"/>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Rashee Rice</t>
-        </is>
-      </c>
+      <c r="D49" s="8" t="n"/>
       <c r="E49" s="8" t="n"/>
       <c r="F49" s="8" t="n"/>
       <c r="G49" s="8" t="n"/>
@@ -12168,7 +12168,7 @@
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>Bucky Irving</t>
+          <t>Chuba Hubbard</t>
         </is>
       </c>
       <c r="C50" s="8" t="n"/>
@@ -12180,11 +12180,11 @@
     </row>
     <row r="51">
       <c r="A51" s="7" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>Chuba Hubbard</t>
+          <t>Quinshon Judkins</t>
         </is>
       </c>
       <c r="C51" s="8" t="n"/>
@@ -13208,7 +13208,7 @@
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
@@ -13596,7 +13596,7 @@
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>Omarion Hampton</t>
+          <t>D'Andre Swift</t>
         </is>
       </c>
       <c r="C28" s="8" t="n"/>
@@ -13610,13 +13610,13 @@
       <c r="A29" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="B29" s="8" t="n"/>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Omarion Hampton</t>
+        </is>
+      </c>
       <c r="C29" s="8" t="n"/>
-      <c r="D29" s="8" t="inlineStr">
-        <is>
-          <t>George Pickens</t>
-        </is>
-      </c>
+      <c r="D29" s="8" t="n"/>
       <c r="E29" s="8" t="n"/>
       <c r="F29" s="8" t="n"/>
       <c r="G29" s="8" t="n"/>
@@ -13630,7 +13630,7 @@
       <c r="C30" s="8" t="n"/>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>DeVonta Smith</t>
+          <t>George Pickens</t>
         </is>
       </c>
       <c r="E30" s="8" t="n"/>
@@ -13644,43 +13644,43 @@
       </c>
       <c r="B31" s="8" t="n"/>
       <c r="C31" s="8" t="n"/>
-      <c r="D31" s="8" t="n"/>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>DeVonta Smith</t>
+        </is>
+      </c>
       <c r="E31" s="8" t="n"/>
       <c r="F31" s="8" t="n"/>
       <c r="G31" s="8" t="n"/>
-      <c r="H31" s="8" t="inlineStr">
-        <is>
-          <t>Josh Allen</t>
-        </is>
-      </c>
+      <c r="H31" s="8" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B32" s="8" t="n"/>
       <c r="C32" s="8" t="n"/>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>A.J. Brown</t>
-        </is>
-      </c>
+      <c r="D32" s="8" t="n"/>
       <c r="E32" s="8" t="n"/>
       <c r="F32" s="8" t="n"/>
       <c r="G32" s="8" t="n"/>
-      <c r="H32" s="8" t="n"/>
+      <c r="H32" s="8" t="inlineStr">
+        <is>
+          <t>Josh Allen</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="B33" s="8" t="inlineStr">
-        <is>
-          <t>D'Andre Swift</t>
-        </is>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="B33" s="8" t="n"/>
       <c r="C33" s="8" t="n"/>
-      <c r="D33" s="8" t="n"/>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>A.J. Brown</t>
+        </is>
+      </c>
       <c r="E33" s="8" t="n"/>
       <c r="F33" s="8" t="n"/>
       <c r="G33" s="8" t="n"/>
@@ -13834,13 +13834,13 @@
       <c r="A43" s="7" t="n">
         <v>24</v>
       </c>
-      <c r="B43" s="8" t="inlineStr">
-        <is>
-          <t>Cam Skattebo</t>
-        </is>
-      </c>
+      <c r="B43" s="8" t="n"/>
       <c r="C43" s="8" t="n"/>
-      <c r="D43" s="8" t="n"/>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Rashee Rice</t>
+        </is>
+      </c>
       <c r="E43" s="8" t="n"/>
       <c r="F43" s="8" t="n"/>
       <c r="G43" s="8" t="n"/>
@@ -13848,15 +13848,15 @@
     </row>
     <row r="44">
       <c r="A44" s="7" t="n">
-        <v>24</v>
-      </c>
-      <c r="B44" s="8" t="n"/>
+        <v>23</v>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>Jeremiyah Love</t>
+        </is>
+      </c>
       <c r="C44" s="8" t="n"/>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Rashee Rice</t>
-        </is>
-      </c>
+      <c r="D44" s="8" t="n"/>
       <c r="E44" s="8" t="n"/>
       <c r="F44" s="8" t="n"/>
       <c r="G44" s="8" t="n"/>
@@ -13868,7 +13868,7 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>Jeremiyah Love</t>
+          <t>Cam Skattebo</t>
         </is>
       </c>
       <c r="C45" s="8" t="n"/>
@@ -13960,11 +13960,11 @@
     </row>
     <row r="51">
       <c r="A51" s="7" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>Quinshon Judkins</t>
+          <t>Chuba Hubbard</t>
         </is>
       </c>
       <c r="C51" s="8" t="n"/>
@@ -13976,11 +13976,11 @@
     </row>
     <row r="52">
       <c r="A52" s="7" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>Chuba Hubbard</t>
+          <t>Quinshon Judkins</t>
         </is>
       </c>
       <c r="C52" s="8" t="n"/>
@@ -14988,7 +14988,7 @@
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
@@ -15374,13 +15374,13 @@
       <c r="A28" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="B28" s="8" t="n"/>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>D'Andre Swift</t>
+        </is>
+      </c>
       <c r="C28" s="8" t="n"/>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>DeVonta Smith</t>
-        </is>
-      </c>
+      <c r="D28" s="8" t="n"/>
       <c r="E28" s="8" t="n"/>
       <c r="F28" s="8" t="n"/>
       <c r="G28" s="8" t="n"/>
@@ -15420,47 +15420,47 @@
     </row>
     <row r="31">
       <c r="A31" s="7" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B31" s="8" t="n"/>
       <c r="C31" s="8" t="n"/>
-      <c r="D31" s="8" t="n"/>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>DeVonta Smith</t>
+        </is>
+      </c>
       <c r="E31" s="8" t="n"/>
       <c r="F31" s="8" t="n"/>
       <c r="G31" s="8" t="n"/>
-      <c r="H31" s="8" t="inlineStr">
-        <is>
-          <t>Josh Allen</t>
-        </is>
-      </c>
+      <c r="H31" s="8" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B32" s="8" t="n"/>
       <c r="C32" s="8" t="n"/>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>A.J. Brown</t>
-        </is>
-      </c>
+      <c r="D32" s="8" t="n"/>
       <c r="E32" s="8" t="n"/>
       <c r="F32" s="8" t="n"/>
       <c r="G32" s="8" t="n"/>
-      <c r="H32" s="8" t="n"/>
+      <c r="H32" s="8" t="inlineStr">
+        <is>
+          <t>Josh Allen</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n">
-        <v>29</v>
-      </c>
-      <c r="B33" s="8" t="inlineStr">
-        <is>
-          <t>D'Andre Swift</t>
-        </is>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="B33" s="8" t="n"/>
       <c r="C33" s="8" t="n"/>
-      <c r="D33" s="8" t="n"/>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>A.J. Brown</t>
+        </is>
+      </c>
       <c r="E33" s="8" t="n"/>
       <c r="F33" s="8" t="n"/>
       <c r="G33" s="8" t="n"/>
@@ -15614,13 +15614,13 @@
       <c r="A43" s="7" t="n">
         <v>22</v>
       </c>
-      <c r="B43" s="8" t="inlineStr">
-        <is>
-          <t>Cam Skattebo</t>
-        </is>
-      </c>
+      <c r="B43" s="8" t="n"/>
       <c r="C43" s="8" t="n"/>
-      <c r="D43" s="8" t="n"/>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Tee Higgins</t>
+        </is>
+      </c>
       <c r="E43" s="8" t="n"/>
       <c r="F43" s="8" t="n"/>
       <c r="G43" s="8" t="n"/>
@@ -15634,7 +15634,7 @@
       <c r="C44" s="8" t="n"/>
       <c r="D44" s="8" t="inlineStr">
         <is>
-          <t>Tee Higgins</t>
+          <t>Tetairoa McMillan</t>
         </is>
       </c>
       <c r="E44" s="8" t="n"/>
@@ -15650,7 +15650,7 @@
       <c r="C45" s="8" t="n"/>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>Tetairoa McMillan</t>
+          <t>Rashee Rice</t>
         </is>
       </c>
       <c r="E45" s="8" t="n"/>
@@ -15660,15 +15660,15 @@
     </row>
     <row r="46">
       <c r="A46" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="B46" s="8" t="n"/>
+        <v>21</v>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>Jeremiyah Love</t>
+        </is>
+      </c>
       <c r="C46" s="8" t="n"/>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>Rashee Rice</t>
-        </is>
-      </c>
+      <c r="D46" s="8" t="n"/>
       <c r="E46" s="8" t="n"/>
       <c r="F46" s="8" t="n"/>
       <c r="G46" s="8" t="n"/>
@@ -15680,7 +15680,7 @@
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>Jeremiyah Love</t>
+          <t>Cam Skattebo</t>
         </is>
       </c>
       <c r="C47" s="8" t="n"/>
@@ -15740,11 +15740,11 @@
     </row>
     <row r="51">
       <c r="A51" s="7" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>Quinshon Judkins</t>
+          <t>Chuba Hubbard</t>
         </is>
       </c>
       <c r="C51" s="8" t="n"/>
@@ -15756,11 +15756,11 @@
     </row>
     <row r="52">
       <c r="A52" s="7" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>Chuba Hubbard</t>
+          <t>Quinshon Judkins</t>
         </is>
       </c>
       <c r="C52" s="8" t="n"/>

</xml_diff>

<commit_message>
Overrides pin the published Half PPR 10-team value after the re-seed
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TradeValueSheets/TradeValues_AllCombinations.xlsx
+++ b/TradeValueSheets/TradeValues_AllCombinations.xlsx
@@ -1020,7 +1020,7 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B21" s="8" t="n"/>
       <c r="C21" s="8" t="n"/>
@@ -1052,33 +1052,33 @@
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
-        <v>34</v>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>Breece Hall</t>
-        </is>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="B23" s="8" t="n"/>
       <c r="C23" s="8" t="n"/>
       <c r="D23" s="8" t="n"/>
       <c r="E23" s="8" t="n"/>
       <c r="F23" s="8" t="n"/>
       <c r="G23" s="8" t="n"/>
-      <c r="H23" s="8" t="n"/>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>Josh Allen</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B24" s="8" t="n"/>
       <c r="C24" s="8" t="n"/>
-      <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>Garrett Wilson</t>
-        </is>
-      </c>
+      <c r="D24" s="8" t="n"/>
       <c r="E24" s="8" t="n"/>
-      <c r="F24" s="8" t="n"/>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Brock Bowers</t>
+        </is>
+      </c>
       <c r="G24" s="8" t="n"/>
       <c r="H24" s="8" t="n"/>
     </row>
@@ -1086,27 +1086,27 @@
       <c r="A25" s="7" t="n">
         <v>34</v>
       </c>
-      <c r="B25" s="8" t="n"/>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Breece Hall</t>
+        </is>
+      </c>
       <c r="C25" s="8" t="n"/>
       <c r="D25" s="8" t="n"/>
       <c r="E25" s="8" t="n"/>
       <c r="F25" s="8" t="n"/>
       <c r="G25" s="8" t="n"/>
-      <c r="H25" s="8" t="inlineStr">
-        <is>
-          <t>Josh Allen</t>
-        </is>
-      </c>
+      <c r="H25" s="8" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B26" s="8" t="n"/>
       <c r="C26" s="8" t="n"/>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>Nico Collins</t>
+          <t>Garrett Wilson</t>
         </is>
       </c>
       <c r="E26" s="8" t="n"/>
@@ -1120,13 +1120,13 @@
       </c>
       <c r="B27" s="8" t="n"/>
       <c r="C27" s="8" t="n"/>
-      <c r="D27" s="8" t="n"/>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Nico Collins</t>
+        </is>
+      </c>
       <c r="E27" s="8" t="n"/>
-      <c r="F27" s="8" t="inlineStr">
-        <is>
-          <t>Brock Bowers</t>
-        </is>
-      </c>
+      <c r="F27" s="8" t="n"/>
       <c r="G27" s="8" t="n"/>
       <c r="H27" s="8" t="n"/>
     </row>
@@ -2736,7 +2736,7 @@
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B18" s="8" t="n"/>
       <c r="C18" s="8" t="n"/>
@@ -2800,17 +2800,17 @@
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B22" s="8" t="n"/>
       <c r="C22" s="8" t="n"/>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Drake London</t>
-        </is>
-      </c>
+      <c r="D22" s="8" t="n"/>
       <c r="E22" s="8" t="n"/>
-      <c r="F22" s="8" t="n"/>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Trey McBride</t>
+        </is>
+      </c>
       <c r="G22" s="8" t="n"/>
       <c r="H22" s="8" t="n"/>
     </row>
@@ -2820,45 +2820,45 @@
       </c>
       <c r="B23" s="8" t="n"/>
       <c r="C23" s="8" t="n"/>
-      <c r="D23" s="8" t="n"/>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Drake London</t>
+        </is>
+      </c>
       <c r="E23" s="8" t="n"/>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>Trey McBride</t>
-        </is>
-      </c>
+      <c r="F23" s="8" t="n"/>
       <c r="G23" s="8" t="n"/>
       <c r="H23" s="8" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
-        <v>34</v>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>Breece Hall</t>
-        </is>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="B24" s="8" t="n"/>
       <c r="C24" s="8" t="n"/>
       <c r="D24" s="8" t="n"/>
       <c r="E24" s="8" t="n"/>
-      <c r="F24" s="8" t="n"/>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Brock Bowers</t>
+        </is>
+      </c>
       <c r="G24" s="8" t="n"/>
       <c r="H24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
-        <v>32</v>
-      </c>
-      <c r="B25" s="8" t="n"/>
+        <v>34</v>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Breece Hall</t>
+        </is>
+      </c>
       <c r="C25" s="8" t="n"/>
       <c r="D25" s="8" t="n"/>
       <c r="E25" s="8" t="n"/>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>Brock Bowers</t>
-        </is>
-      </c>
+      <c r="F25" s="8" t="n"/>
       <c r="G25" s="8" t="n"/>
       <c r="H25" s="8" t="n"/>
     </row>
@@ -3488,31 +3488,31 @@
     </row>
     <row r="65">
       <c r="A65" s="7" t="n">
-        <v>11</v>
-      </c>
-      <c r="B65" s="8" t="inlineStr">
-        <is>
-          <t>David Montgomery</t>
-        </is>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="B65" s="8" t="n"/>
       <c r="C65" s="8" t="n"/>
       <c r="D65" s="8" t="n"/>
       <c r="E65" s="8" t="n"/>
       <c r="F65" s="8" t="n"/>
       <c r="G65" s="8" t="n"/>
-      <c r="H65" s="8" t="n"/>
+      <c r="H65" s="8" t="inlineStr">
+        <is>
+          <t>Drake Maye</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="B66" s="8" t="n"/>
+      <c r="B66" s="8" t="inlineStr">
+        <is>
+          <t>David Montgomery</t>
+        </is>
+      </c>
       <c r="C66" s="8" t="n"/>
-      <c r="D66" s="8" t="inlineStr">
-        <is>
-          <t>Emeka Egbuka</t>
-        </is>
-      </c>
+      <c r="D66" s="8" t="n"/>
       <c r="E66" s="8" t="n"/>
       <c r="F66" s="8" t="n"/>
       <c r="G66" s="8" t="n"/>
@@ -3524,13 +3524,13 @@
       </c>
       <c r="B67" s="8" t="n"/>
       <c r="C67" s="8" t="n"/>
-      <c r="D67" s="8" t="n"/>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>Emeka Egbuka</t>
+        </is>
+      </c>
       <c r="E67" s="8" t="n"/>
-      <c r="F67" s="8" t="inlineStr">
-        <is>
-          <t>Isaiah Likely</t>
-        </is>
-      </c>
+      <c r="F67" s="8" t="n"/>
       <c r="G67" s="8" t="n"/>
       <c r="H67" s="8" t="n"/>
     </row>
@@ -3542,13 +3542,13 @@
       <c r="C68" s="8" t="n"/>
       <c r="D68" s="8" t="n"/>
       <c r="E68" s="8" t="n"/>
-      <c r="F68" s="8" t="n"/>
+      <c r="F68" s="8" t="inlineStr">
+        <is>
+          <t>Isaiah Likely</t>
+        </is>
+      </c>
       <c r="G68" s="8" t="n"/>
-      <c r="H68" s="8" t="inlineStr">
-        <is>
-          <t>Drake Maye</t>
-        </is>
-      </c>
+      <c r="H68" s="8" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="n">
@@ -4484,35 +4484,35 @@
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
-        <v>43</v>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Saquon Barkley</t>
-        </is>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="B17" s="8" t="n"/>
       <c r="C17" s="8" t="n"/>
       <c r="D17" s="8" t="n"/>
       <c r="E17" s="8" t="n"/>
       <c r="F17" s="8" t="n"/>
       <c r="G17" s="8" t="n"/>
-      <c r="H17" s="8" t="n"/>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>Josh Allen</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
-        <v>42</v>
-      </c>
-      <c r="B18" s="8" t="n"/>
+        <v>43</v>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Saquon Barkley</t>
+        </is>
+      </c>
       <c r="C18" s="8" t="n"/>
       <c r="D18" s="8" t="n"/>
       <c r="E18" s="8" t="n"/>
       <c r="F18" s="8" t="n"/>
       <c r="G18" s="8" t="n"/>
-      <c r="H18" s="8" t="inlineStr">
-        <is>
-          <t>Josh Allen</t>
-        </is>
-      </c>
+      <c r="H18" s="8" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
@@ -4564,17 +4564,17 @@
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B22" s="8" t="n"/>
       <c r="C22" s="8" t="n"/>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Drake London</t>
-        </is>
-      </c>
+      <c r="D22" s="8" t="n"/>
       <c r="E22" s="8" t="n"/>
-      <c r="F22" s="8" t="n"/>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Trey McBride</t>
+        </is>
+      </c>
       <c r="G22" s="8" t="n"/>
       <c r="H22" s="8" t="n"/>
     </row>
@@ -4584,45 +4584,45 @@
       </c>
       <c r="B23" s="8" t="n"/>
       <c r="C23" s="8" t="n"/>
-      <c r="D23" s="8" t="n"/>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Drake London</t>
+        </is>
+      </c>
       <c r="E23" s="8" t="n"/>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>Trey McBride</t>
-        </is>
-      </c>
+      <c r="F23" s="8" t="n"/>
       <c r="G23" s="8" t="n"/>
       <c r="H23" s="8" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
-        <v>33</v>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>Breece Hall</t>
-        </is>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="B24" s="8" t="n"/>
       <c r="C24" s="8" t="n"/>
       <c r="D24" s="8" t="n"/>
       <c r="E24" s="8" t="n"/>
-      <c r="F24" s="8" t="n"/>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Brock Bowers</t>
+        </is>
+      </c>
       <c r="G24" s="8" t="n"/>
       <c r="H24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
-        <v>31</v>
-      </c>
-      <c r="B25" s="8" t="n"/>
+        <v>33</v>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Breece Hall</t>
+        </is>
+      </c>
       <c r="C25" s="8" t="n"/>
       <c r="D25" s="8" t="n"/>
       <c r="E25" s="8" t="n"/>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>Brock Bowers</t>
-        </is>
-      </c>
+      <c r="F25" s="8" t="n"/>
       <c r="G25" s="8" t="n"/>
       <c r="H25" s="8" t="n"/>
     </row>
@@ -5252,19 +5252,19 @@
     </row>
     <row r="65">
       <c r="A65" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="B65" s="8" t="inlineStr">
-        <is>
-          <t>David Montgomery</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B65" s="8" t="n"/>
       <c r="C65" s="8" t="n"/>
       <c r="D65" s="8" t="n"/>
       <c r="E65" s="8" t="n"/>
       <c r="F65" s="8" t="n"/>
       <c r="G65" s="8" t="n"/>
-      <c r="H65" s="8" t="n"/>
+      <c r="H65" s="8" t="inlineStr">
+        <is>
+          <t>Drake Maye</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="n">
@@ -5272,7 +5272,7 @@
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>Jordan Mason</t>
+          <t>David Montgomery</t>
         </is>
       </c>
       <c r="C66" s="8" t="n"/>
@@ -5288,7 +5288,7 @@
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>J.K. Dobbins</t>
+          <t>Jordan Mason</t>
         </is>
       </c>
       <c r="C67" s="8" t="n"/>
@@ -5304,7 +5304,7 @@
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>Jacory Croskey-Merritt</t>
+          <t>J.K. Dobbins</t>
         </is>
       </c>
       <c r="C68" s="8" t="n"/>
@@ -5318,13 +5318,13 @@
       <c r="A69" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B69" s="8" t="n"/>
+      <c r="B69" s="8" t="inlineStr">
+        <is>
+          <t>Jacory Croskey-Merritt</t>
+        </is>
+      </c>
       <c r="C69" s="8" t="n"/>
-      <c r="D69" s="8" t="inlineStr">
-        <is>
-          <t>Emeka Egbuka</t>
-        </is>
-      </c>
+      <c r="D69" s="8" t="n"/>
       <c r="E69" s="8" t="n"/>
       <c r="F69" s="8" t="n"/>
       <c r="G69" s="8" t="n"/>
@@ -5336,13 +5336,13 @@
       </c>
       <c r="B70" s="8" t="n"/>
       <c r="C70" s="8" t="n"/>
-      <c r="D70" s="8" t="n"/>
+      <c r="D70" s="8" t="inlineStr">
+        <is>
+          <t>Emeka Egbuka</t>
+        </is>
+      </c>
       <c r="E70" s="8" t="n"/>
-      <c r="F70" s="8" t="inlineStr">
-        <is>
-          <t>Isaiah Likely</t>
-        </is>
-      </c>
+      <c r="F70" s="8" t="n"/>
       <c r="G70" s="8" t="n"/>
       <c r="H70" s="8" t="n"/>
     </row>
@@ -5354,13 +5354,13 @@
       <c r="C71" s="8" t="n"/>
       <c r="D71" s="8" t="n"/>
       <c r="E71" s="8" t="n"/>
-      <c r="F71" s="8" t="n"/>
+      <c r="F71" s="8" t="inlineStr">
+        <is>
+          <t>Isaiah Likely</t>
+        </is>
+      </c>
       <c r="G71" s="8" t="n"/>
-      <c r="H71" s="8" t="inlineStr">
-        <is>
-          <t>Drake Maye</t>
-        </is>
-      </c>
+      <c r="H71" s="8" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="n">
@@ -6248,35 +6248,35 @@
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
-        <v>43</v>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Saquon Barkley</t>
-        </is>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="B17" s="8" t="n"/>
       <c r="C17" s="8" t="n"/>
       <c r="D17" s="8" t="n"/>
       <c r="E17" s="8" t="n"/>
       <c r="F17" s="8" t="n"/>
       <c r="G17" s="8" t="n"/>
-      <c r="H17" s="8" t="n"/>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>Josh Allen</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
-        <v>41</v>
-      </c>
-      <c r="B18" s="8" t="n"/>
+        <v>43</v>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Saquon Barkley</t>
+        </is>
+      </c>
       <c r="C18" s="8" t="n"/>
       <c r="D18" s="8" t="n"/>
       <c r="E18" s="8" t="n"/>
       <c r="F18" s="8" t="n"/>
       <c r="G18" s="8" t="n"/>
-      <c r="H18" s="8" t="inlineStr">
-        <is>
-          <t>Josh Allen</t>
-        </is>
-      </c>
+      <c r="H18" s="8" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
@@ -6328,17 +6328,17 @@
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B22" s="8" t="n"/>
       <c r="C22" s="8" t="n"/>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Drake London</t>
-        </is>
-      </c>
+      <c r="D22" s="8" t="n"/>
       <c r="E22" s="8" t="n"/>
-      <c r="F22" s="8" t="n"/>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Trey McBride</t>
+        </is>
+      </c>
       <c r="G22" s="8" t="n"/>
       <c r="H22" s="8" t="n"/>
     </row>
@@ -6348,45 +6348,45 @@
       </c>
       <c r="B23" s="8" t="n"/>
       <c r="C23" s="8" t="n"/>
-      <c r="D23" s="8" t="n"/>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Drake London</t>
+        </is>
+      </c>
       <c r="E23" s="8" t="n"/>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>Trey McBride</t>
-        </is>
-      </c>
+      <c r="F23" s="8" t="n"/>
       <c r="G23" s="8" t="n"/>
       <c r="H23" s="8" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
-        <v>32</v>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>Breece Hall</t>
-        </is>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="B24" s="8" t="n"/>
       <c r="C24" s="8" t="n"/>
       <c r="D24" s="8" t="n"/>
       <c r="E24" s="8" t="n"/>
-      <c r="F24" s="8" t="n"/>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Brock Bowers</t>
+        </is>
+      </c>
       <c r="G24" s="8" t="n"/>
       <c r="H24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
-        <v>29</v>
-      </c>
-      <c r="B25" s="8" t="n"/>
+        <v>32</v>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Breece Hall</t>
+        </is>
+      </c>
       <c r="C25" s="8" t="n"/>
       <c r="D25" s="8" t="n"/>
       <c r="E25" s="8" t="n"/>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>Brock Bowers</t>
-        </is>
-      </c>
+      <c r="F25" s="8" t="n"/>
       <c r="G25" s="8" t="n"/>
       <c r="H25" s="8" t="n"/>
     </row>
@@ -8076,7 +8076,7 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B21" s="8" t="n"/>
       <c r="C21" s="8" t="n"/>
@@ -8092,7 +8092,7 @@
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B22" s="8" t="n"/>
       <c r="C22" s="8" t="n"/>
@@ -8124,31 +8124,31 @@
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
-        <v>35</v>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>Breece Hall</t>
-        </is>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="B24" s="8" t="n"/>
       <c r="C24" s="8" t="n"/>
       <c r="D24" s="8" t="n"/>
       <c r="E24" s="8" t="n"/>
-      <c r="F24" s="8" t="n"/>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Brock Bowers</t>
+        </is>
+      </c>
       <c r="G24" s="8" t="n"/>
       <c r="H24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
-        <v>33</v>
-      </c>
-      <c r="B25" s="8" t="n"/>
+        <v>35</v>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Breece Hall</t>
+        </is>
+      </c>
       <c r="C25" s="8" t="n"/>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>Garrett Wilson</t>
-        </is>
-      </c>
+      <c r="D25" s="8" t="n"/>
       <c r="E25" s="8" t="n"/>
       <c r="F25" s="8" t="n"/>
       <c r="G25" s="8" t="n"/>
@@ -8160,13 +8160,13 @@
       </c>
       <c r="B26" s="8" t="n"/>
       <c r="C26" s="8" t="n"/>
-      <c r="D26" s="8" t="n"/>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Garrett Wilson</t>
+        </is>
+      </c>
       <c r="E26" s="8" t="n"/>
-      <c r="F26" s="8" t="inlineStr">
-        <is>
-          <t>Brock Bowers</t>
-        </is>
-      </c>
+      <c r="F26" s="8" t="n"/>
       <c r="G26" s="8" t="n"/>
       <c r="H26" s="8" t="n"/>
     </row>
@@ -8940,19 +8940,19 @@
     </row>
     <row r="75">
       <c r="A75" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B75" s="8" t="n"/>
       <c r="C75" s="8" t="n"/>
       <c r="D75" s="8" t="n"/>
       <c r="E75" s="8" t="n"/>
-      <c r="F75" s="8" t="inlineStr">
-        <is>
-          <t>Isaiah Likely</t>
-        </is>
-      </c>
+      <c r="F75" s="8" t="n"/>
       <c r="G75" s="8" t="n"/>
-      <c r="H75" s="8" t="n"/>
+      <c r="H75" s="8" t="inlineStr">
+        <is>
+          <t>Drake Maye</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="7" t="n">
@@ -8962,13 +8962,13 @@
       <c r="C76" s="8" t="n"/>
       <c r="D76" s="8" t="n"/>
       <c r="E76" s="8" t="n"/>
-      <c r="F76" s="8" t="n"/>
+      <c r="F76" s="8" t="inlineStr">
+        <is>
+          <t>Isaiah Likely</t>
+        </is>
+      </c>
       <c r="G76" s="8" t="n"/>
-      <c r="H76" s="8" t="inlineStr">
-        <is>
-          <t>Drake Maye</t>
-        </is>
-      </c>
+      <c r="H76" s="8" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="n">
@@ -9840,7 +9840,7 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B21" s="8" t="n"/>
       <c r="C21" s="8" t="n"/>
@@ -9856,7 +9856,7 @@
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B22" s="8" t="n"/>
       <c r="C22" s="8" t="n"/>
@@ -9888,31 +9888,31 @@
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
-        <v>34</v>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>Breece Hall</t>
-        </is>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="B24" s="8" t="n"/>
       <c r="C24" s="8" t="n"/>
       <c r="D24" s="8" t="n"/>
       <c r="E24" s="8" t="n"/>
-      <c r="F24" s="8" t="n"/>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Brock Bowers</t>
+        </is>
+      </c>
       <c r="G24" s="8" t="n"/>
       <c r="H24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
-        <v>32</v>
-      </c>
-      <c r="B25" s="8" t="n"/>
+        <v>34</v>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Breece Hall</t>
+        </is>
+      </c>
       <c r="C25" s="8" t="n"/>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>Garrett Wilson</t>
-        </is>
-      </c>
+      <c r="D25" s="8" t="n"/>
       <c r="E25" s="8" t="n"/>
       <c r="F25" s="8" t="n"/>
       <c r="G25" s="8" t="n"/>
@@ -9924,13 +9924,13 @@
       </c>
       <c r="B26" s="8" t="n"/>
       <c r="C26" s="8" t="n"/>
-      <c r="D26" s="8" t="n"/>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Garrett Wilson</t>
+        </is>
+      </c>
       <c r="E26" s="8" t="n"/>
-      <c r="F26" s="8" t="inlineStr">
-        <is>
-          <t>Brock Bowers</t>
-        </is>
-      </c>
+      <c r="F26" s="8" t="n"/>
       <c r="G26" s="8" t="n"/>
       <c r="H26" s="8" t="n"/>
     </row>
@@ -10704,19 +10704,19 @@
     </row>
     <row r="75">
       <c r="A75" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B75" s="8" t="inlineStr">
-        <is>
-          <t>Rhamondre Stevenson</t>
-        </is>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="B75" s="8" t="n"/>
       <c r="C75" s="8" t="n"/>
       <c r="D75" s="8" t="n"/>
       <c r="E75" s="8" t="n"/>
       <c r="F75" s="8" t="n"/>
       <c r="G75" s="8" t="n"/>
-      <c r="H75" s="8" t="n"/>
+      <c r="H75" s="8" t="inlineStr">
+        <is>
+          <t>Drake Maye</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="7" t="n">
@@ -10724,7 +10724,7 @@
       </c>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>Jordan Mason</t>
+          <t>Rhamondre Stevenson</t>
         </is>
       </c>
       <c r="C76" s="8" t="n"/>
@@ -10740,7 +10740,7 @@
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>J.K. Dobbins</t>
+          <t>Jordan Mason</t>
         </is>
       </c>
       <c r="C77" s="8" t="n"/>
@@ -10756,7 +10756,7 @@
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>Jacory Croskey-Merritt</t>
+          <t>J.K. Dobbins</t>
         </is>
       </c>
       <c r="C78" s="8" t="n"/>
@@ -10770,13 +10770,13 @@
       <c r="A79" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B79" s="8" t="n"/>
+      <c r="B79" s="8" t="inlineStr">
+        <is>
+          <t>Jacory Croskey-Merritt</t>
+        </is>
+      </c>
       <c r="C79" s="8" t="n"/>
-      <c r="D79" s="8" t="inlineStr">
-        <is>
-          <t>Carnell Tate</t>
-        </is>
-      </c>
+      <c r="D79" s="8" t="n"/>
       <c r="E79" s="8" t="n"/>
       <c r="F79" s="8" t="n"/>
       <c r="G79" s="8" t="n"/>
@@ -10790,7 +10790,7 @@
       <c r="C80" s="8" t="n"/>
       <c r="D80" s="8" t="inlineStr">
         <is>
-          <t>Alec Pierce</t>
+          <t>Carnell Tate</t>
         </is>
       </c>
       <c r="E80" s="8" t="n"/>
@@ -10804,13 +10804,13 @@
       </c>
       <c r="B81" s="8" t="n"/>
       <c r="C81" s="8" t="n"/>
-      <c r="D81" s="8" t="n"/>
+      <c r="D81" s="8" t="inlineStr">
+        <is>
+          <t>Alec Pierce</t>
+        </is>
+      </c>
       <c r="E81" s="8" t="n"/>
-      <c r="F81" s="8" t="inlineStr">
-        <is>
-          <t>Isaiah Likely</t>
-        </is>
-      </c>
+      <c r="F81" s="8" t="n"/>
       <c r="G81" s="8" t="n"/>
       <c r="H81" s="8" t="n"/>
     </row>
@@ -10822,13 +10822,13 @@
       <c r="C82" s="8" t="n"/>
       <c r="D82" s="8" t="n"/>
       <c r="E82" s="8" t="n"/>
-      <c r="F82" s="8" t="n"/>
+      <c r="F82" s="8" t="inlineStr">
+        <is>
+          <t>Isaiah Likely</t>
+        </is>
+      </c>
       <c r="G82" s="8" t="n"/>
-      <c r="H82" s="8" t="inlineStr">
-        <is>
-          <t>Drake Maye</t>
-        </is>
-      </c>
+      <c r="H82" s="8" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="n">
@@ -11604,7 +11604,7 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B21" s="8" t="n"/>
       <c r="C21" s="8" t="n"/>
@@ -11620,7 +11620,7 @@
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B22" s="8" t="n"/>
       <c r="C22" s="8" t="n"/>
@@ -11652,31 +11652,31 @@
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
-        <v>33</v>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>Breece Hall</t>
-        </is>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="B24" s="8" t="n"/>
       <c r="C24" s="8" t="n"/>
       <c r="D24" s="8" t="n"/>
       <c r="E24" s="8" t="n"/>
-      <c r="F24" s="8" t="n"/>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Brock Bowers</t>
+        </is>
+      </c>
       <c r="G24" s="8" t="n"/>
       <c r="H24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
-        <v>31</v>
-      </c>
-      <c r="B25" s="8" t="n"/>
+        <v>33</v>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Breece Hall</t>
+        </is>
+      </c>
       <c r="C25" s="8" t="n"/>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>Garrett Wilson</t>
-        </is>
-      </c>
+      <c r="D25" s="8" t="n"/>
       <c r="E25" s="8" t="n"/>
       <c r="F25" s="8" t="n"/>
       <c r="G25" s="8" t="n"/>
@@ -11688,13 +11688,13 @@
       </c>
       <c r="B26" s="8" t="n"/>
       <c r="C26" s="8" t="n"/>
-      <c r="D26" s="8" t="n"/>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Garrett Wilson</t>
+        </is>
+      </c>
       <c r="E26" s="8" t="n"/>
-      <c r="F26" s="8" t="inlineStr">
-        <is>
-          <t>Brock Bowers</t>
-        </is>
-      </c>
+      <c r="F26" s="8" t="n"/>
       <c r="G26" s="8" t="n"/>
       <c r="H26" s="8" t="n"/>
     </row>
@@ -13368,7 +13368,7 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B21" s="8" t="n"/>
       <c r="C21" s="8" t="n"/>
@@ -13400,47 +13400,47 @@
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B23" s="8" t="n"/>
       <c r="C23" s="8" t="n"/>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>Garrett Wilson</t>
-        </is>
-      </c>
+      <c r="D23" s="8" t="n"/>
       <c r="E23" s="8" t="n"/>
       <c r="F23" s="8" t="n"/>
       <c r="G23" s="8" t="n"/>
-      <c r="H23" s="8" t="n"/>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>Josh Allen</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B24" s="8" t="n"/>
       <c r="C24" s="8" t="n"/>
       <c r="D24" s="8" t="n"/>
       <c r="E24" s="8" t="n"/>
-      <c r="F24" s="8" t="n"/>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Brock Bowers</t>
+        </is>
+      </c>
       <c r="G24" s="8" t="n"/>
-      <c r="H24" s="8" t="inlineStr">
-        <is>
-          <t>Josh Allen</t>
-        </is>
-      </c>
+      <c r="H24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
-        <v>35</v>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>Breece Hall</t>
-        </is>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="B25" s="8" t="n"/>
       <c r="C25" s="8" t="n"/>
-      <c r="D25" s="8" t="n"/>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Garrett Wilson</t>
+        </is>
+      </c>
       <c r="E25" s="8" t="n"/>
       <c r="F25" s="8" t="n"/>
       <c r="G25" s="8" t="n"/>
@@ -13448,15 +13448,15 @@
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
-        <v>34</v>
-      </c>
-      <c r="B26" s="8" t="n"/>
+        <v>35</v>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>Breece Hall</t>
+        </is>
+      </c>
       <c r="C26" s="8" t="n"/>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>Nico Collins</t>
-        </is>
-      </c>
+      <c r="D26" s="8" t="n"/>
       <c r="E26" s="8" t="n"/>
       <c r="F26" s="8" t="n"/>
       <c r="G26" s="8" t="n"/>
@@ -13468,13 +13468,13 @@
       </c>
       <c r="B27" s="8" t="n"/>
       <c r="C27" s="8" t="n"/>
-      <c r="D27" s="8" t="n"/>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Nico Collins</t>
+        </is>
+      </c>
       <c r="E27" s="8" t="n"/>
-      <c r="F27" s="8" t="inlineStr">
-        <is>
-          <t>Brock Bowers</t>
-        </is>
-      </c>
+      <c r="F27" s="8" t="n"/>
       <c r="G27" s="8" t="n"/>
       <c r="H27" s="8" t="n"/>
     </row>
@@ -14376,33 +14376,33 @@
     </row>
     <row r="84">
       <c r="A84" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B84" s="8" t="inlineStr">
-        <is>
-          <t>Rachaad White</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="B84" s="8" t="n"/>
       <c r="C84" s="8" t="n"/>
       <c r="D84" s="8" t="n"/>
       <c r="E84" s="8" t="n"/>
       <c r="F84" s="8" t="n"/>
       <c r="G84" s="8" t="n"/>
-      <c r="H84" s="8" t="n"/>
+      <c r="H84" s="8" t="inlineStr">
+        <is>
+          <t>Drake Maye</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B85" s="8" t="n"/>
+      <c r="B85" s="8" t="inlineStr">
+        <is>
+          <t>Rachaad White</t>
+        </is>
+      </c>
       <c r="C85" s="8" t="n"/>
       <c r="D85" s="8" t="n"/>
       <c r="E85" s="8" t="n"/>
-      <c r="F85" s="8" t="inlineStr">
-        <is>
-          <t>Isaiah Likely</t>
-        </is>
-      </c>
+      <c r="F85" s="8" t="n"/>
       <c r="G85" s="8" t="n"/>
       <c r="H85" s="8" t="n"/>
     </row>
@@ -14414,13 +14414,13 @@
       <c r="C86" s="8" t="n"/>
       <c r="D86" s="8" t="n"/>
       <c r="E86" s="8" t="n"/>
-      <c r="F86" s="8" t="n"/>
+      <c r="F86" s="8" t="inlineStr">
+        <is>
+          <t>Isaiah Likely</t>
+        </is>
+      </c>
       <c r="G86" s="8" t="n"/>
-      <c r="H86" s="8" t="inlineStr">
-        <is>
-          <t>Drake Maye</t>
-        </is>
-      </c>
+      <c r="H86" s="8" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="n">
@@ -15132,7 +15132,7 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B21" s="8" t="n"/>
       <c r="C21" s="8" t="n"/>
@@ -15164,33 +15164,33 @@
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
-        <v>35</v>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>Breece Hall</t>
-        </is>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="B23" s="8" t="n"/>
       <c r="C23" s="8" t="n"/>
       <c r="D23" s="8" t="n"/>
       <c r="E23" s="8" t="n"/>
       <c r="F23" s="8" t="n"/>
       <c r="G23" s="8" t="n"/>
-      <c r="H23" s="8" t="n"/>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>Josh Allen</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B24" s="8" t="n"/>
       <c r="C24" s="8" t="n"/>
-      <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>Garrett Wilson</t>
-        </is>
-      </c>
+      <c r="D24" s="8" t="n"/>
       <c r="E24" s="8" t="n"/>
-      <c r="F24" s="8" t="n"/>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Brock Bowers</t>
+        </is>
+      </c>
       <c r="G24" s="8" t="n"/>
       <c r="H24" s="8" t="n"/>
     </row>
@@ -15198,27 +15198,27 @@
       <c r="A25" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="B25" s="8" t="n"/>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Breece Hall</t>
+        </is>
+      </c>
       <c r="C25" s="8" t="n"/>
       <c r="D25" s="8" t="n"/>
       <c r="E25" s="8" t="n"/>
       <c r="F25" s="8" t="n"/>
       <c r="G25" s="8" t="n"/>
-      <c r="H25" s="8" t="inlineStr">
-        <is>
-          <t>Josh Allen</t>
-        </is>
-      </c>
+      <c r="H25" s="8" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B26" s="8" t="n"/>
       <c r="C26" s="8" t="n"/>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>Nico Collins</t>
+          <t>Garrett Wilson</t>
         </is>
       </c>
       <c r="E26" s="8" t="n"/>
@@ -15232,13 +15232,13 @@
       </c>
       <c r="B27" s="8" t="n"/>
       <c r="C27" s="8" t="n"/>
-      <c r="D27" s="8" t="n"/>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Nico Collins</t>
+        </is>
+      </c>
       <c r="E27" s="8" t="n"/>
-      <c r="F27" s="8" t="inlineStr">
-        <is>
-          <t>Brock Bowers</t>
-        </is>
-      </c>
+      <c r="F27" s="8" t="n"/>
       <c r="G27" s="8" t="n"/>
       <c r="H27" s="8" t="n"/>
     </row>
@@ -16124,31 +16124,31 @@
     </row>
     <row r="83">
       <c r="A83" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="B83" s="8" t="inlineStr">
-        <is>
-          <t>Rachaad White</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="B83" s="8" t="n"/>
       <c r="C83" s="8" t="n"/>
       <c r="D83" s="8" t="n"/>
       <c r="E83" s="8" t="n"/>
       <c r="F83" s="8" t="n"/>
       <c r="G83" s="8" t="n"/>
-      <c r="H83" s="8" t="n"/>
+      <c r="H83" s="8" t="inlineStr">
+        <is>
+          <t>Drake Maye</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B84" s="8" t="n"/>
+      <c r="B84" s="8" t="inlineStr">
+        <is>
+          <t>Rachaad White</t>
+        </is>
+      </c>
       <c r="C84" s="8" t="n"/>
-      <c r="D84" s="8" t="inlineStr">
-        <is>
-          <t>DK Metcalf</t>
-        </is>
-      </c>
+      <c r="D84" s="8" t="n"/>
       <c r="E84" s="8" t="n"/>
       <c r="F84" s="8" t="n"/>
       <c r="G84" s="8" t="n"/>
@@ -16160,13 +16160,13 @@
       </c>
       <c r="B85" s="8" t="n"/>
       <c r="C85" s="8" t="n"/>
-      <c r="D85" s="8" t="n"/>
+      <c r="D85" s="8" t="inlineStr">
+        <is>
+          <t>DK Metcalf</t>
+        </is>
+      </c>
       <c r="E85" s="8" t="n"/>
-      <c r="F85" s="8" t="inlineStr">
-        <is>
-          <t>Isaiah Likely</t>
-        </is>
-      </c>
+      <c r="F85" s="8" t="n"/>
       <c r="G85" s="8" t="n"/>
       <c r="H85" s="8" t="n"/>
     </row>
@@ -16178,13 +16178,13 @@
       <c r="C86" s="8" t="n"/>
       <c r="D86" s="8" t="n"/>
       <c r="E86" s="8" t="n"/>
-      <c r="F86" s="8" t="n"/>
+      <c r="F86" s="8" t="inlineStr">
+        <is>
+          <t>Isaiah Likely</t>
+        </is>
+      </c>
       <c r="G86" s="8" t="n"/>
-      <c r="H86" s="8" t="inlineStr">
-        <is>
-          <t>Drake Maye</t>
-        </is>
-      </c>
+      <c r="H86" s="8" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="n">

</xml_diff>

<commit_message>
Revert "Update trade value sheets"
This reverts commit e1501b656f195de8e75896a81c88101a87c892e5.
</commit_message>
<xml_diff>
--- a/TradeValueSheets/TradeValues_AllCombinations.xlsx
+++ b/TradeValueSheets/TradeValues_AllCombinations.xlsx
@@ -1040,29 +1040,29 @@
       </c>
       <c r="B22" s="8" t="n"/>
       <c r="C22" s="8" t="n"/>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Chris Olave</t>
-        </is>
-      </c>
+      <c r="D22" s="8" t="n"/>
       <c r="E22" s="8" t="n"/>
-      <c r="F22" s="8" t="n"/>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Trey McBride</t>
+        </is>
+      </c>
       <c r="G22" s="8" t="n"/>
       <c r="H22" s="8" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B23" s="8" t="n"/>
       <c r="C23" s="8" t="n"/>
-      <c r="D23" s="8" t="n"/>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Chris Olave</t>
+        </is>
+      </c>
       <c r="E23" s="8" t="n"/>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>Trey McBride</t>
-        </is>
-      </c>
+      <c r="F23" s="8" t="n"/>
       <c r="G23" s="8" t="n"/>
       <c r="H23" s="8" t="n"/>
     </row>
@@ -1234,7 +1234,7 @@
       <c r="C34" s="8" t="n"/>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>A.J. Brown</t>
+          <t>Mike Evans</t>
         </is>
       </c>
       <c r="E34" s="8" t="n"/>
@@ -1250,7 +1250,7 @@
       <c r="C35" s="8" t="n"/>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>Garrett Wilson</t>
+          <t>A.J. Brown</t>
         </is>
       </c>
       <c r="E35" s="8" t="n"/>
@@ -1260,13 +1260,13 @@
     </row>
     <row r="36">
       <c r="A36" s="7" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B36" s="8" t="n"/>
       <c r="C36" s="8" t="n"/>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>Mike Evans</t>
+          <t>Garrett Wilson</t>
         </is>
       </c>
       <c r="E36" s="8" t="n"/>
@@ -1666,7 +1666,7 @@
       <c r="C61" s="8" t="n"/>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>Terry McLaurin</t>
+          <t>Michael Wilson</t>
         </is>
       </c>
       <c r="E61" s="8" t="n"/>
@@ -1676,15 +1676,15 @@
     </row>
     <row r="62">
       <c r="A62" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="B62" s="8" t="n"/>
+        <v>7</v>
+      </c>
+      <c r="B62" s="8" t="inlineStr">
+        <is>
+          <t>MarShawn Lloyd</t>
+        </is>
+      </c>
       <c r="C62" s="8" t="n"/>
-      <c r="D62" s="8" t="inlineStr">
-        <is>
-          <t>Michael Wilson</t>
-        </is>
-      </c>
+      <c r="D62" s="8" t="n"/>
       <c r="E62" s="8" t="n"/>
       <c r="F62" s="8" t="n"/>
       <c r="G62" s="8" t="n"/>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>MarShawn Lloyd</t>
+          <t>David Montgomery</t>
         </is>
       </c>
       <c r="C63" s="8" t="n"/>
@@ -1710,13 +1710,13 @@
       <c r="A64" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B64" s="8" t="inlineStr">
-        <is>
-          <t>David Montgomery</t>
-        </is>
-      </c>
+      <c r="B64" s="8" t="n"/>
       <c r="C64" s="8" t="n"/>
-      <c r="D64" s="8" t="n"/>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>DJ Moore</t>
+        </is>
+      </c>
       <c r="E64" s="8" t="n"/>
       <c r="F64" s="8" t="n"/>
       <c r="G64" s="8" t="n"/>
@@ -1730,7 +1730,7 @@
       <c r="C65" s="8" t="n"/>
       <c r="D65" s="8" t="inlineStr">
         <is>
-          <t>DJ Moore</t>
+          <t>Jameson Williams</t>
         </is>
       </c>
       <c r="E65" s="8" t="n"/>
@@ -1746,7 +1746,7 @@
       <c r="C66" s="8" t="n"/>
       <c r="D66" s="8" t="inlineStr">
         <is>
-          <t>Jameson Williams</t>
+          <t>Terry McLaurin</t>
         </is>
       </c>
       <c r="E66" s="8" t="n"/>
@@ -1836,17 +1836,17 @@
     </row>
     <row r="72">
       <c r="A72" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B72" s="8" t="inlineStr">
-        <is>
-          <t>Rachaad White</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="B72" s="8" t="n"/>
       <c r="C72" s="8" t="n"/>
       <c r="D72" s="8" t="n"/>
       <c r="E72" s="8" t="n"/>
-      <c r="F72" s="8" t="n"/>
+      <c r="F72" s="8" t="inlineStr">
+        <is>
+          <t>Isaiah Likely</t>
+        </is>
+      </c>
       <c r="G72" s="8" t="n"/>
       <c r="H72" s="8" t="n"/>
     </row>
@@ -1854,13 +1854,13 @@
       <c r="A73" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B73" s="8" t="n"/>
+      <c r="B73" s="8" t="inlineStr">
+        <is>
+          <t>Rachaad White</t>
+        </is>
+      </c>
       <c r="C73" s="8" t="n"/>
-      <c r="D73" s="8" t="inlineStr">
-        <is>
-          <t>Alec Pierce</t>
-        </is>
-      </c>
+      <c r="D73" s="8" t="n"/>
       <c r="E73" s="8" t="n"/>
       <c r="F73" s="8" t="n"/>
       <c r="G73" s="8" t="n"/>
@@ -1872,13 +1872,13 @@
       </c>
       <c r="B74" s="8" t="n"/>
       <c r="C74" s="8" t="n"/>
-      <c r="D74" s="8" t="n"/>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>Alec Pierce</t>
+        </is>
+      </c>
       <c r="E74" s="8" t="n"/>
-      <c r="F74" s="8" t="inlineStr">
-        <is>
-          <t>Isaiah Likely</t>
-        </is>
-      </c>
+      <c r="F74" s="8" t="n"/>
       <c r="G74" s="8" t="n"/>
       <c r="H74" s="8" t="n"/>
     </row>
@@ -2848,7 +2848,7 @@
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B25" s="8" t="n"/>
       <c r="C25" s="8" t="n"/>
@@ -2992,13 +2992,13 @@
     </row>
     <row r="34">
       <c r="A34" s="7" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B34" s="8" t="n"/>
       <c r="C34" s="8" t="n"/>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>DeVonta Smith</t>
+          <t>Mike Evans</t>
         </is>
       </c>
       <c r="E34" s="8" t="n"/>
@@ -3014,7 +3014,7 @@
       <c r="C35" s="8" t="n"/>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>A.J. Brown</t>
+          <t>DeVonta Smith</t>
         </is>
       </c>
       <c r="E35" s="8" t="n"/>
@@ -3030,7 +3030,7 @@
       <c r="C36" s="8" t="n"/>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>Mike Evans</t>
+          <t>A.J. Brown</t>
         </is>
       </c>
       <c r="E36" s="8" t="n"/>
@@ -3874,13 +3874,13 @@
       <c r="A89" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B89" s="8" t="n"/>
+      <c r="B89" s="8" t="inlineStr">
+        <is>
+          <t>Jacory Croskey-Merritt</t>
+        </is>
+      </c>
       <c r="C89" s="8" t="n"/>
-      <c r="D89" s="8" t="inlineStr">
-        <is>
-          <t>Terry McLaurin</t>
-        </is>
-      </c>
+      <c r="D89" s="8" t="n"/>
       <c r="E89" s="8" t="n"/>
       <c r="F89" s="8" t="n"/>
       <c r="G89" s="8" t="n"/>
@@ -3986,13 +3986,13 @@
       <c r="A96" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B96" s="8" t="inlineStr">
-        <is>
-          <t>Jacory Croskey-Merritt</t>
-        </is>
-      </c>
+      <c r="B96" s="8" t="n"/>
       <c r="C96" s="8" t="n"/>
-      <c r="D96" s="8" t="n"/>
+      <c r="D96" s="8" t="inlineStr">
+        <is>
+          <t>Terry McLaurin</t>
+        </is>
+      </c>
       <c r="E96" s="8" t="n"/>
       <c r="F96" s="8" t="n"/>
       <c r="G96" s="8" t="n"/>
@@ -4612,7 +4612,7 @@
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B25" s="8" t="n"/>
       <c r="C25" s="8" t="n"/>
@@ -4756,13 +4756,13 @@
     </row>
     <row r="34">
       <c r="A34" s="7" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B34" s="8" t="n"/>
       <c r="C34" s="8" t="n"/>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>A.J. Brown</t>
+          <t>Mike Evans</t>
         </is>
       </c>
       <c r="E34" s="8" t="n"/>
@@ -4772,13 +4772,13 @@
     </row>
     <row r="35">
       <c r="A35" s="7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B35" s="8" t="n"/>
       <c r="C35" s="8" t="n"/>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>DeVonta Smith</t>
+          <t>A.J. Brown</t>
         </is>
       </c>
       <c r="E35" s="8" t="n"/>
@@ -4794,7 +4794,7 @@
       <c r="C36" s="8" t="n"/>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>Mike Evans</t>
+          <t>DeVonta Smith</t>
         </is>
       </c>
       <c r="E36" s="8" t="n"/>
@@ -5562,7 +5562,7 @@
       <c r="C84" s="8" t="n"/>
       <c r="D84" s="8" t="inlineStr">
         <is>
-          <t>Terry McLaurin</t>
+          <t>Michael Wilson</t>
         </is>
       </c>
       <c r="E84" s="8" t="n"/>
@@ -5578,7 +5578,7 @@
       <c r="C85" s="8" t="n"/>
       <c r="D85" s="8" t="inlineStr">
         <is>
-          <t>Michael Wilson</t>
+          <t>De'Zhaun Stribling</t>
         </is>
       </c>
       <c r="E85" s="8" t="n"/>
@@ -5594,7 +5594,7 @@
       <c r="C86" s="8" t="n"/>
       <c r="D86" s="8" t="inlineStr">
         <is>
-          <t>De'Zhaun Stribling</t>
+          <t>Quentin Johnston</t>
         </is>
       </c>
       <c r="E86" s="8" t="n"/>
@@ -5604,15 +5604,15 @@
     </row>
     <row r="87">
       <c r="A87" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="B87" s="8" t="n"/>
+        <v>6</v>
+      </c>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>David Montgomery</t>
+        </is>
+      </c>
       <c r="C87" s="8" t="n"/>
-      <c r="D87" s="8" t="inlineStr">
-        <is>
-          <t>Quentin Johnston</t>
-        </is>
-      </c>
+      <c r="D87" s="8" t="n"/>
       <c r="E87" s="8" t="n"/>
       <c r="F87" s="8" t="n"/>
       <c r="G87" s="8" t="n"/>
@@ -5624,7 +5624,7 @@
       </c>
       <c r="B88" s="8" t="inlineStr">
         <is>
-          <t>David Montgomery</t>
+          <t>J.K. Dobbins</t>
         </is>
       </c>
       <c r="C88" s="8" t="n"/>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="B89" s="8" t="inlineStr">
         <is>
-          <t>J.K. Dobbins</t>
+          <t>Blake Corum</t>
         </is>
       </c>
       <c r="C89" s="8" t="n"/>
@@ -5656,7 +5656,7 @@
       </c>
       <c r="B90" s="8" t="inlineStr">
         <is>
-          <t>Blake Corum</t>
+          <t>Jacory Croskey-Merritt</t>
         </is>
       </c>
       <c r="C90" s="8" t="n"/>
@@ -5674,7 +5674,7 @@
       <c r="C91" s="8" t="n"/>
       <c r="D91" s="8" t="inlineStr">
         <is>
-          <t>Chris Godwin Jr.</t>
+          <t>Terry McLaurin</t>
         </is>
       </c>
       <c r="E91" s="8" t="n"/>
@@ -5688,13 +5688,13 @@
       </c>
       <c r="B92" s="8" t="n"/>
       <c r="C92" s="8" t="n"/>
-      <c r="D92" s="8" t="n"/>
+      <c r="D92" s="8" t="inlineStr">
+        <is>
+          <t>Chris Godwin Jr.</t>
+        </is>
+      </c>
       <c r="E92" s="8" t="n"/>
-      <c r="F92" s="8" t="inlineStr">
-        <is>
-          <t>Harold Fannin Jr.</t>
-        </is>
-      </c>
+      <c r="F92" s="8" t="n"/>
       <c r="G92" s="8" t="n"/>
       <c r="H92" s="8" t="n"/>
     </row>
@@ -5706,13 +5706,13 @@
       <c r="C93" s="8" t="n"/>
       <c r="D93" s="8" t="n"/>
       <c r="E93" s="8" t="n"/>
-      <c r="F93" s="8" t="n"/>
+      <c r="F93" s="8" t="inlineStr">
+        <is>
+          <t>Harold Fannin Jr.</t>
+        </is>
+      </c>
       <c r="G93" s="8" t="n"/>
-      <c r="H93" s="8" t="inlineStr">
-        <is>
-          <t>Jalen Hurts</t>
-        </is>
-      </c>
+      <c r="H93" s="8" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="n">
@@ -5726,7 +5726,7 @@
       <c r="G94" s="8" t="n"/>
       <c r="H94" s="8" t="inlineStr">
         <is>
-          <t>Justin Herbert</t>
+          <t>Jalen Hurts</t>
         </is>
       </c>
     </row>
@@ -5742,25 +5742,25 @@
       <c r="G95" s="8" t="n"/>
       <c r="H95" s="8" t="inlineStr">
         <is>
-          <t>Trevor Lawrence</t>
+          <t>Justin Herbert</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B96" s="8" t="inlineStr">
-        <is>
-          <t>Jacory Croskey-Merritt</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="B96" s="8" t="n"/>
       <c r="C96" s="8" t="n"/>
       <c r="D96" s="8" t="n"/>
       <c r="E96" s="8" t="n"/>
       <c r="F96" s="8" t="n"/>
       <c r="G96" s="8" t="n"/>
-      <c r="H96" s="8" t="n"/>
+      <c r="H96" s="8" t="inlineStr">
+        <is>
+          <t>Trevor Lawrence</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="7" t="n">
@@ -6376,7 +6376,7 @@
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B25" s="8" t="n"/>
       <c r="C25" s="8" t="n"/>
@@ -6520,13 +6520,13 @@
     </row>
     <row r="34">
       <c r="A34" s="7" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B34" s="8" t="n"/>
       <c r="C34" s="8" t="n"/>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>DeVonta Smith</t>
+          <t>Mike Evans</t>
         </is>
       </c>
       <c r="E34" s="8" t="n"/>
@@ -6542,7 +6542,7 @@
       <c r="C35" s="8" t="n"/>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>A.J. Brown</t>
+          <t>DeVonta Smith</t>
         </is>
       </c>
       <c r="E35" s="8" t="n"/>
@@ -6558,7 +6558,7 @@
       <c r="C36" s="8" t="n"/>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>Mike Evans</t>
+          <t>A.J. Brown</t>
         </is>
       </c>
       <c r="E36" s="8" t="n"/>
@@ -6776,17 +6776,17 @@
     </row>
     <row r="50">
       <c r="A50" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="B50" s="8" t="inlineStr">
-        <is>
-          <t>Bucky Irving</t>
-        </is>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="B50" s="8" t="n"/>
       <c r="C50" s="8" t="n"/>
       <c r="D50" s="8" t="n"/>
       <c r="E50" s="8" t="n"/>
-      <c r="F50" s="8" t="n"/>
+      <c r="F50" s="8" t="inlineStr">
+        <is>
+          <t>Isaiah Likely</t>
+        </is>
+      </c>
       <c r="G50" s="8" t="n"/>
       <c r="H50" s="8" t="n"/>
     </row>
@@ -6794,15 +6794,15 @@
       <c r="A51" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="B51" s="8" t="n"/>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>Bucky Irving</t>
+        </is>
+      </c>
       <c r="C51" s="8" t="n"/>
       <c r="D51" s="8" t="n"/>
       <c r="E51" s="8" t="n"/>
-      <c r="F51" s="8" t="inlineStr">
-        <is>
-          <t>Isaiah Likely</t>
-        </is>
-      </c>
+      <c r="F51" s="8" t="n"/>
       <c r="G51" s="8" t="n"/>
       <c r="H51" s="8" t="n"/>
     </row>
@@ -7370,13 +7370,13 @@
       <c r="A87" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B87" s="8" t="n"/>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>Jacory Croskey-Merritt</t>
+        </is>
+      </c>
       <c r="C87" s="8" t="n"/>
-      <c r="D87" s="8" t="inlineStr">
-        <is>
-          <t>Terry McLaurin</t>
-        </is>
-      </c>
+      <c r="D87" s="8" t="n"/>
       <c r="E87" s="8" t="n"/>
       <c r="F87" s="8" t="n"/>
       <c r="G87" s="8" t="n"/>
@@ -7514,13 +7514,13 @@
       <c r="A96" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B96" s="8" t="inlineStr">
-        <is>
-          <t>Jacory Croskey-Merritt</t>
-        </is>
-      </c>
+      <c r="B96" s="8" t="n"/>
       <c r="C96" s="8" t="n"/>
-      <c r="D96" s="8" t="n"/>
+      <c r="D96" s="8" t="inlineStr">
+        <is>
+          <t>Terry McLaurin</t>
+        </is>
+      </c>
       <c r="E96" s="8" t="n"/>
       <c r="F96" s="8" t="n"/>
       <c r="G96" s="8" t="n"/>
@@ -8140,7 +8140,7 @@
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B25" s="8" t="n"/>
       <c r="C25" s="8" t="n"/>
@@ -8268,13 +8268,13 @@
     </row>
     <row r="33">
       <c r="A33" s="7" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B33" s="8" t="n"/>
       <c r="C33" s="8" t="n"/>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>A.J. Brown</t>
+          <t>Mike Evans</t>
         </is>
       </c>
       <c r="E33" s="8" t="n"/>
@@ -8290,7 +8290,7 @@
       <c r="C34" s="8" t="n"/>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>Rashee Rice</t>
+          <t>A.J. Brown</t>
         </is>
       </c>
       <c r="E34" s="8" t="n"/>
@@ -8300,15 +8300,15 @@
     </row>
     <row r="35">
       <c r="A35" s="7" t="n">
-        <v>25</v>
-      </c>
-      <c r="B35" s="8" t="inlineStr">
-        <is>
-          <t>Omarion Hampton</t>
-        </is>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="B35" s="8" t="n"/>
       <c r="C35" s="8" t="n"/>
-      <c r="D35" s="8" t="n"/>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Rashee Rice</t>
+        </is>
+      </c>
       <c r="E35" s="8" t="n"/>
       <c r="F35" s="8" t="n"/>
       <c r="G35" s="8" t="n"/>
@@ -8318,13 +8318,13 @@
       <c r="A36" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="B36" s="8" t="n"/>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>Omarion Hampton</t>
+        </is>
+      </c>
       <c r="C36" s="8" t="n"/>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>Garrett Wilson</t>
-        </is>
-      </c>
+      <c r="D36" s="8" t="n"/>
       <c r="E36" s="8" t="n"/>
       <c r="F36" s="8" t="n"/>
       <c r="G36" s="8" t="n"/>
@@ -8336,31 +8336,31 @@
       </c>
       <c r="B37" s="8" t="n"/>
       <c r="C37" s="8" t="n"/>
-      <c r="D37" s="8" t="n"/>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Garrett Wilson</t>
+        </is>
+      </c>
       <c r="E37" s="8" t="n"/>
       <c r="F37" s="8" t="n"/>
       <c r="G37" s="8" t="n"/>
-      <c r="H37" s="8" t="inlineStr">
-        <is>
-          <t>Lamar Jackson</t>
-        </is>
-      </c>
+      <c r="H37" s="8" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B38" s="8" t="n"/>
       <c r="C38" s="8" t="n"/>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Mike Evans</t>
-        </is>
-      </c>
+      <c r="D38" s="8" t="n"/>
       <c r="E38" s="8" t="n"/>
       <c r="F38" s="8" t="n"/>
       <c r="G38" s="8" t="n"/>
-      <c r="H38" s="8" t="n"/>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
+          <t>Lamar Jackson</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n">
@@ -8684,17 +8684,17 @@
     </row>
     <row r="59">
       <c r="A59" s="7" t="n">
-        <v>13</v>
-      </c>
-      <c r="B59" s="8" t="inlineStr">
-        <is>
-          <t>Rhamondre Stevenson</t>
-        </is>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="B59" s="8" t="n"/>
       <c r="C59" s="8" t="n"/>
       <c r="D59" s="8" t="n"/>
       <c r="E59" s="8" t="n"/>
-      <c r="F59" s="8" t="n"/>
+      <c r="F59" s="8" t="inlineStr">
+        <is>
+          <t>Isaiah Likely</t>
+        </is>
+      </c>
       <c r="G59" s="8" t="n"/>
       <c r="H59" s="8" t="n"/>
     </row>
@@ -8702,15 +8702,15 @@
       <c r="A60" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="B60" s="8" t="n"/>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>Rhamondre Stevenson</t>
+        </is>
+      </c>
       <c r="C60" s="8" t="n"/>
       <c r="D60" s="8" t="n"/>
       <c r="E60" s="8" t="n"/>
-      <c r="F60" s="8" t="inlineStr">
-        <is>
-          <t>Isaiah Likely</t>
-        </is>
-      </c>
+      <c r="F60" s="8" t="n"/>
       <c r="G60" s="8" t="n"/>
       <c r="H60" s="8" t="n"/>
     </row>
@@ -8850,7 +8850,7 @@
       <c r="C69" s="8" t="n"/>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>Terry McLaurin</t>
+          <t>Jameson Williams</t>
         </is>
       </c>
       <c r="E69" s="8" t="n"/>
@@ -8866,7 +8866,7 @@
       <c r="C70" s="8" t="n"/>
       <c r="D70" s="8" t="inlineStr">
         <is>
-          <t>Jameson Williams</t>
+          <t>Michael Wilson</t>
         </is>
       </c>
       <c r="E70" s="8" t="n"/>
@@ -8876,15 +8876,15 @@
     </row>
     <row r="71">
       <c r="A71" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="B71" s="8" t="n"/>
+        <v>9</v>
+      </c>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>David Montgomery</t>
+        </is>
+      </c>
       <c r="C71" s="8" t="n"/>
-      <c r="D71" s="8" t="inlineStr">
-        <is>
-          <t>Michael Wilson</t>
-        </is>
-      </c>
+      <c r="D71" s="8" t="n"/>
       <c r="E71" s="8" t="n"/>
       <c r="F71" s="8" t="n"/>
       <c r="G71" s="8" t="n"/>
@@ -8896,7 +8896,7 @@
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>David Montgomery</t>
+          <t>Josh Jacobs</t>
         </is>
       </c>
       <c r="C72" s="8" t="n"/>
@@ -8910,13 +8910,13 @@
       <c r="A73" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B73" s="8" t="inlineStr">
-        <is>
-          <t>Josh Jacobs</t>
-        </is>
-      </c>
+      <c r="B73" s="8" t="n"/>
       <c r="C73" s="8" t="n"/>
-      <c r="D73" s="8" t="n"/>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <t>Terry McLaurin</t>
+        </is>
+      </c>
       <c r="E73" s="8" t="n"/>
       <c r="F73" s="8" t="n"/>
       <c r="G73" s="8" t="n"/>
@@ -9326,13 +9326,13 @@
       <c r="A99" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B99" s="8" t="n"/>
+      <c r="B99" s="8" t="inlineStr">
+        <is>
+          <t>Jacory Croskey-Merritt</t>
+        </is>
+      </c>
       <c r="C99" s="8" t="n"/>
-      <c r="D99" s="8" t="inlineStr">
-        <is>
-          <t>Chris Godwin Jr.</t>
-        </is>
-      </c>
+      <c r="D99" s="8" t="n"/>
       <c r="E99" s="8" t="n"/>
       <c r="F99" s="8" t="n"/>
       <c r="G99" s="8" t="n"/>
@@ -9344,13 +9344,13 @@
       </c>
       <c r="B100" s="8" t="n"/>
       <c r="C100" s="8" t="n"/>
-      <c r="D100" s="8" t="n"/>
+      <c r="D100" s="8" t="inlineStr">
+        <is>
+          <t>Chris Godwin Jr.</t>
+        </is>
+      </c>
       <c r="E100" s="8" t="n"/>
-      <c r="F100" s="8" t="inlineStr">
-        <is>
-          <t>Harold Fannin Jr.</t>
-        </is>
-      </c>
+      <c r="F100" s="8" t="n"/>
       <c r="G100" s="8" t="n"/>
       <c r="H100" s="8" t="n"/>
     </row>
@@ -9362,13 +9362,13 @@
       <c r="C101" s="8" t="n"/>
       <c r="D101" s="8" t="n"/>
       <c r="E101" s="8" t="n"/>
-      <c r="F101" s="8" t="n"/>
+      <c r="F101" s="8" t="inlineStr">
+        <is>
+          <t>Harold Fannin Jr.</t>
+        </is>
+      </c>
       <c r="G101" s="8" t="n"/>
-      <c r="H101" s="8" t="inlineStr">
-        <is>
-          <t>Jalen Hurts</t>
-        </is>
-      </c>
+      <c r="H101" s="8" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="n">
@@ -9382,7 +9382,7 @@
       <c r="G102" s="8" t="n"/>
       <c r="H102" s="8" t="inlineStr">
         <is>
-          <t>Justin Herbert</t>
+          <t>Jalen Hurts</t>
         </is>
       </c>
     </row>
@@ -9398,25 +9398,25 @@
       <c r="G103" s="8" t="n"/>
       <c r="H103" s="8" t="inlineStr">
         <is>
-          <t>Trevor Lawrence</t>
+          <t>Justin Herbert</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="B104" s="8" t="inlineStr">
-        <is>
-          <t>Jacory Croskey-Merritt</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="B104" s="8" t="n"/>
       <c r="C104" s="8" t="n"/>
       <c r="D104" s="8" t="n"/>
       <c r="E104" s="8" t="n"/>
       <c r="F104" s="8" t="n"/>
       <c r="G104" s="8" t="n"/>
-      <c r="H104" s="8" t="n"/>
+      <c r="H104" s="8" t="inlineStr">
+        <is>
+          <t>Trevor Lawrence</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="n">
@@ -9904,7 +9904,7 @@
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B25" s="8" t="n"/>
       <c r="C25" s="8" t="n"/>
@@ -10032,13 +10032,13 @@
     </row>
     <row r="33">
       <c r="A33" s="7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B33" s="8" t="n"/>
       <c r="C33" s="8" t="n"/>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>A.J. Brown</t>
+          <t>Mike Evans</t>
         </is>
       </c>
       <c r="E33" s="8" t="n"/>
@@ -10054,7 +10054,7 @@
       <c r="C34" s="8" t="n"/>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>Rashee Rice</t>
+          <t>A.J. Brown</t>
         </is>
       </c>
       <c r="E34" s="8" t="n"/>
@@ -10064,15 +10064,15 @@
     </row>
     <row r="35">
       <c r="A35" s="7" t="n">
-        <v>23</v>
-      </c>
-      <c r="B35" s="8" t="inlineStr">
-        <is>
-          <t>Omarion Hampton</t>
-        </is>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="B35" s="8" t="n"/>
       <c r="C35" s="8" t="n"/>
-      <c r="D35" s="8" t="n"/>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Rashee Rice</t>
+        </is>
+      </c>
       <c r="E35" s="8" t="n"/>
       <c r="F35" s="8" t="n"/>
       <c r="G35" s="8" t="n"/>
@@ -10082,13 +10082,13 @@
       <c r="A36" s="7" t="n">
         <v>23</v>
       </c>
-      <c r="B36" s="8" t="n"/>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>Omarion Hampton</t>
+        </is>
+      </c>
       <c r="C36" s="8" t="n"/>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>Garrett Wilson</t>
-        </is>
-      </c>
+      <c r="D36" s="8" t="n"/>
       <c r="E36" s="8" t="n"/>
       <c r="F36" s="8" t="n"/>
       <c r="G36" s="8" t="n"/>
@@ -10100,31 +10100,31 @@
       </c>
       <c r="B37" s="8" t="n"/>
       <c r="C37" s="8" t="n"/>
-      <c r="D37" s="8" t="n"/>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Garrett Wilson</t>
+        </is>
+      </c>
       <c r="E37" s="8" t="n"/>
       <c r="F37" s="8" t="n"/>
       <c r="G37" s="8" t="n"/>
-      <c r="H37" s="8" t="inlineStr">
-        <is>
-          <t>Lamar Jackson</t>
-        </is>
-      </c>
+      <c r="H37" s="8" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B38" s="8" t="n"/>
       <c r="C38" s="8" t="n"/>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Mike Evans</t>
-        </is>
-      </c>
+      <c r="D38" s="8" t="n"/>
       <c r="E38" s="8" t="n"/>
       <c r="F38" s="8" t="n"/>
       <c r="G38" s="8" t="n"/>
-      <c r="H38" s="8" t="n"/>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
+          <t>Lamar Jackson</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n">
@@ -10448,17 +10448,17 @@
     </row>
     <row r="59">
       <c r="A59" s="7" t="n">
-        <v>11</v>
-      </c>
-      <c r="B59" s="8" t="inlineStr">
-        <is>
-          <t>Rhamondre Stevenson</t>
-        </is>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="B59" s="8" t="n"/>
       <c r="C59" s="8" t="n"/>
       <c r="D59" s="8" t="n"/>
       <c r="E59" s="8" t="n"/>
-      <c r="F59" s="8" t="n"/>
+      <c r="F59" s="8" t="inlineStr">
+        <is>
+          <t>Isaiah Likely</t>
+        </is>
+      </c>
       <c r="G59" s="8" t="n"/>
       <c r="H59" s="8" t="n"/>
     </row>
@@ -10466,15 +10466,15 @@
       <c r="A60" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="B60" s="8" t="n"/>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>Rhamondre Stevenson</t>
+        </is>
+      </c>
       <c r="C60" s="8" t="n"/>
       <c r="D60" s="8" t="n"/>
       <c r="E60" s="8" t="n"/>
-      <c r="F60" s="8" t="inlineStr">
-        <is>
-          <t>Isaiah Likely</t>
-        </is>
-      </c>
+      <c r="F60" s="8" t="n"/>
       <c r="G60" s="8" t="n"/>
       <c r="H60" s="8" t="n"/>
     </row>
@@ -10614,7 +10614,7 @@
       <c r="C69" s="8" t="n"/>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>Terry McLaurin</t>
+          <t>Jameson Williams</t>
         </is>
       </c>
       <c r="E69" s="8" t="n"/>
@@ -10630,7 +10630,7 @@
       <c r="C70" s="8" t="n"/>
       <c r="D70" s="8" t="inlineStr">
         <is>
-          <t>Jameson Williams</t>
+          <t>Michael Wilson</t>
         </is>
       </c>
       <c r="E70" s="8" t="n"/>
@@ -10640,15 +10640,15 @@
     </row>
     <row r="71">
       <c r="A71" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="B71" s="8" t="n"/>
+        <v>7</v>
+      </c>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>David Montgomery</t>
+        </is>
+      </c>
       <c r="C71" s="8" t="n"/>
-      <c r="D71" s="8" t="inlineStr">
-        <is>
-          <t>Michael Wilson</t>
-        </is>
-      </c>
+      <c r="D71" s="8" t="n"/>
       <c r="E71" s="8" t="n"/>
       <c r="F71" s="8" t="n"/>
       <c r="G71" s="8" t="n"/>
@@ -10660,7 +10660,7 @@
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>David Montgomery</t>
+          <t>Josh Jacobs</t>
         </is>
       </c>
       <c r="C72" s="8" t="n"/>
@@ -10676,7 +10676,7 @@
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>Josh Jacobs</t>
+          <t>TreVeyon Henderson</t>
         </is>
       </c>
       <c r="C73" s="8" t="n"/>
@@ -10692,7 +10692,7 @@
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>TreVeyon Henderson</t>
+          <t>Tony Pollard</t>
         </is>
       </c>
       <c r="C74" s="8" t="n"/>
@@ -10706,13 +10706,13 @@
       <c r="A75" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B75" s="8" t="inlineStr">
-        <is>
-          <t>Tony Pollard</t>
-        </is>
-      </c>
+      <c r="B75" s="8" t="n"/>
       <c r="C75" s="8" t="n"/>
-      <c r="D75" s="8" t="n"/>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>Terry McLaurin</t>
+        </is>
+      </c>
       <c r="E75" s="8" t="n"/>
       <c r="F75" s="8" t="n"/>
       <c r="G75" s="8" t="n"/>
@@ -11090,13 +11090,13 @@
       <c r="A99" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B99" s="8" t="n"/>
+      <c r="B99" s="8" t="inlineStr">
+        <is>
+          <t>Jacory Croskey-Merritt</t>
+        </is>
+      </c>
       <c r="C99" s="8" t="n"/>
-      <c r="D99" s="8" t="inlineStr">
-        <is>
-          <t>Chris Godwin Jr.</t>
-        </is>
-      </c>
+      <c r="D99" s="8" t="n"/>
       <c r="E99" s="8" t="n"/>
       <c r="F99" s="8" t="n"/>
       <c r="G99" s="8" t="n"/>
@@ -11108,13 +11108,13 @@
       </c>
       <c r="B100" s="8" t="n"/>
       <c r="C100" s="8" t="n"/>
-      <c r="D100" s="8" t="n"/>
+      <c r="D100" s="8" t="inlineStr">
+        <is>
+          <t>Chris Godwin Jr.</t>
+        </is>
+      </c>
       <c r="E100" s="8" t="n"/>
-      <c r="F100" s="8" t="inlineStr">
-        <is>
-          <t>Harold Fannin Jr.</t>
-        </is>
-      </c>
+      <c r="F100" s="8" t="n"/>
       <c r="G100" s="8" t="n"/>
       <c r="H100" s="8" t="n"/>
     </row>
@@ -11126,13 +11126,13 @@
       <c r="C101" s="8" t="n"/>
       <c r="D101" s="8" t="n"/>
       <c r="E101" s="8" t="n"/>
-      <c r="F101" s="8" t="n"/>
+      <c r="F101" s="8" t="inlineStr">
+        <is>
+          <t>Harold Fannin Jr.</t>
+        </is>
+      </c>
       <c r="G101" s="8" t="n"/>
-      <c r="H101" s="8" t="inlineStr">
-        <is>
-          <t>Jalen Hurts</t>
-        </is>
-      </c>
+      <c r="H101" s="8" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="n">
@@ -11146,7 +11146,7 @@
       <c r="G102" s="8" t="n"/>
       <c r="H102" s="8" t="inlineStr">
         <is>
-          <t>Justin Herbert</t>
+          <t>Jalen Hurts</t>
         </is>
       </c>
     </row>
@@ -11162,25 +11162,25 @@
       <c r="G103" s="8" t="n"/>
       <c r="H103" s="8" t="inlineStr">
         <is>
-          <t>Trevor Lawrence</t>
+          <t>Justin Herbert</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B104" s="8" t="inlineStr">
-        <is>
-          <t>Jacory Croskey-Merritt</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="B104" s="8" t="n"/>
       <c r="C104" s="8" t="n"/>
       <c r="D104" s="8" t="n"/>
       <c r="E104" s="8" t="n"/>
       <c r="F104" s="8" t="n"/>
       <c r="G104" s="8" t="n"/>
-      <c r="H104" s="8" t="n"/>
+      <c r="H104" s="8" t="inlineStr">
+        <is>
+          <t>Trevor Lawrence</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="n">
@@ -11656,29 +11656,29 @@
       </c>
       <c r="B24" s="8" t="n"/>
       <c r="C24" s="8" t="n"/>
-      <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>Chris Olave</t>
-        </is>
-      </c>
+      <c r="D24" s="8" t="n"/>
       <c r="E24" s="8" t="n"/>
-      <c r="F24" s="8" t="n"/>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Trey McBride</t>
+        </is>
+      </c>
       <c r="G24" s="8" t="n"/>
       <c r="H24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B25" s="8" t="n"/>
       <c r="C25" s="8" t="n"/>
-      <c r="D25" s="8" t="n"/>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Chris Olave</t>
+        </is>
+      </c>
       <c r="E25" s="8" t="n"/>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>Trey McBride</t>
-        </is>
-      </c>
+      <c r="F25" s="8" t="n"/>
       <c r="G25" s="8" t="n"/>
       <c r="H25" s="8" t="n"/>
     </row>
@@ -11796,13 +11796,13 @@
     </row>
     <row r="33">
       <c r="A33" s="7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B33" s="8" t="n"/>
       <c r="C33" s="8" t="n"/>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>A.J. Brown</t>
+          <t>Mike Evans</t>
         </is>
       </c>
       <c r="E33" s="8" t="n"/>
@@ -11818,7 +11818,7 @@
       <c r="C34" s="8" t="n"/>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>Rashee Rice</t>
+          <t>A.J. Brown</t>
         </is>
       </c>
       <c r="E34" s="8" t="n"/>
@@ -11828,15 +11828,15 @@
     </row>
     <row r="35">
       <c r="A35" s="7" t="n">
-        <v>21</v>
-      </c>
-      <c r="B35" s="8" t="inlineStr">
-        <is>
-          <t>Omarion Hampton</t>
-        </is>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="B35" s="8" t="n"/>
       <c r="C35" s="8" t="n"/>
-      <c r="D35" s="8" t="n"/>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Rashee Rice</t>
+        </is>
+      </c>
       <c r="E35" s="8" t="n"/>
       <c r="F35" s="8" t="n"/>
       <c r="G35" s="8" t="n"/>
@@ -11846,13 +11846,13 @@
       <c r="A36" s="7" t="n">
         <v>21</v>
       </c>
-      <c r="B36" s="8" t="n"/>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>Omarion Hampton</t>
+        </is>
+      </c>
       <c r="C36" s="8" t="n"/>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>Garrett Wilson</t>
-        </is>
-      </c>
+      <c r="D36" s="8" t="n"/>
       <c r="E36" s="8" t="n"/>
       <c r="F36" s="8" t="n"/>
       <c r="G36" s="8" t="n"/>
@@ -11864,31 +11864,31 @@
       </c>
       <c r="B37" s="8" t="n"/>
       <c r="C37" s="8" t="n"/>
-      <c r="D37" s="8" t="n"/>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Garrett Wilson</t>
+        </is>
+      </c>
       <c r="E37" s="8" t="n"/>
       <c r="F37" s="8" t="n"/>
       <c r="G37" s="8" t="n"/>
-      <c r="H37" s="8" t="inlineStr">
-        <is>
-          <t>Lamar Jackson</t>
-        </is>
-      </c>
+      <c r="H37" s="8" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B38" s="8" t="n"/>
       <c r="C38" s="8" t="n"/>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Mike Evans</t>
-        </is>
-      </c>
+      <c r="D38" s="8" t="n"/>
       <c r="E38" s="8" t="n"/>
       <c r="F38" s="8" t="n"/>
       <c r="G38" s="8" t="n"/>
-      <c r="H38" s="8" t="n"/>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
+          <t>Lamar Jackson</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n">
@@ -12212,17 +12212,17 @@
     </row>
     <row r="59">
       <c r="A59" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="B59" s="8" t="inlineStr">
-        <is>
-          <t>Rhamondre Stevenson</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B59" s="8" t="n"/>
       <c r="C59" s="8" t="n"/>
       <c r="D59" s="8" t="n"/>
       <c r="E59" s="8" t="n"/>
-      <c r="F59" s="8" t="n"/>
+      <c r="F59" s="8" t="inlineStr">
+        <is>
+          <t>Isaiah Likely</t>
+        </is>
+      </c>
       <c r="G59" s="8" t="n"/>
       <c r="H59" s="8" t="n"/>
     </row>
@@ -12230,15 +12230,15 @@
       <c r="A60" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B60" s="8" t="n"/>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>Rhamondre Stevenson</t>
+        </is>
+      </c>
       <c r="C60" s="8" t="n"/>
       <c r="D60" s="8" t="n"/>
       <c r="E60" s="8" t="n"/>
-      <c r="F60" s="8" t="inlineStr">
-        <is>
-          <t>Isaiah Likely</t>
-        </is>
-      </c>
+      <c r="F60" s="8" t="n"/>
       <c r="G60" s="8" t="n"/>
       <c r="H60" s="8" t="n"/>
     </row>
@@ -12378,7 +12378,7 @@
       <c r="C69" s="8" t="n"/>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>Terry McLaurin</t>
+          <t>Jameson Williams</t>
         </is>
       </c>
       <c r="E69" s="8" t="n"/>
@@ -12394,7 +12394,7 @@
       <c r="C70" s="8" t="n"/>
       <c r="D70" s="8" t="inlineStr">
         <is>
-          <t>Jameson Williams</t>
+          <t>Michael Wilson</t>
         </is>
       </c>
       <c r="E70" s="8" t="n"/>
@@ -12404,15 +12404,15 @@
     </row>
     <row r="71">
       <c r="A71" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="B71" s="8" t="n"/>
+        <v>6</v>
+      </c>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>David Montgomery</t>
+        </is>
+      </c>
       <c r="C71" s="8" t="n"/>
-      <c r="D71" s="8" t="inlineStr">
-        <is>
-          <t>Michael Wilson</t>
-        </is>
-      </c>
+      <c r="D71" s="8" t="n"/>
       <c r="E71" s="8" t="n"/>
       <c r="F71" s="8" t="n"/>
       <c r="G71" s="8" t="n"/>
@@ -12424,7 +12424,7 @@
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>David Montgomery</t>
+          <t>Josh Jacobs</t>
         </is>
       </c>
       <c r="C72" s="8" t="n"/>
@@ -12438,13 +12438,13 @@
       <c r="A73" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B73" s="8" t="inlineStr">
-        <is>
-          <t>Josh Jacobs</t>
-        </is>
-      </c>
+      <c r="B73" s="8" t="n"/>
       <c r="C73" s="8" t="n"/>
-      <c r="D73" s="8" t="n"/>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <t>Terry McLaurin</t>
+        </is>
+      </c>
       <c r="E73" s="8" t="n"/>
       <c r="F73" s="8" t="n"/>
       <c r="G73" s="8" t="n"/>
@@ -12854,13 +12854,13 @@
       <c r="A99" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B99" s="8" t="n"/>
+      <c r="B99" s="8" t="inlineStr">
+        <is>
+          <t>Jacory Croskey-Merritt</t>
+        </is>
+      </c>
       <c r="C99" s="8" t="n"/>
-      <c r="D99" s="8" t="inlineStr">
-        <is>
-          <t>Chris Godwin Jr.</t>
-        </is>
-      </c>
+      <c r="D99" s="8" t="n"/>
       <c r="E99" s="8" t="n"/>
       <c r="F99" s="8" t="n"/>
       <c r="G99" s="8" t="n"/>
@@ -12872,13 +12872,13 @@
       </c>
       <c r="B100" s="8" t="n"/>
       <c r="C100" s="8" t="n"/>
-      <c r="D100" s="8" t="n"/>
+      <c r="D100" s="8" t="inlineStr">
+        <is>
+          <t>Chris Godwin Jr.</t>
+        </is>
+      </c>
       <c r="E100" s="8" t="n"/>
-      <c r="F100" s="8" t="inlineStr">
-        <is>
-          <t>Harold Fannin Jr.</t>
-        </is>
-      </c>
+      <c r="F100" s="8" t="n"/>
       <c r="G100" s="8" t="n"/>
       <c r="H100" s="8" t="n"/>
     </row>
@@ -12890,13 +12890,13 @@
       <c r="C101" s="8" t="n"/>
       <c r="D101" s="8" t="n"/>
       <c r="E101" s="8" t="n"/>
-      <c r="F101" s="8" t="n"/>
+      <c r="F101" s="8" t="inlineStr">
+        <is>
+          <t>Harold Fannin Jr.</t>
+        </is>
+      </c>
       <c r="G101" s="8" t="n"/>
-      <c r="H101" s="8" t="inlineStr">
-        <is>
-          <t>Jalen Hurts</t>
-        </is>
-      </c>
+      <c r="H101" s="8" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="n">
@@ -12910,7 +12910,7 @@
       <c r="G102" s="8" t="n"/>
       <c r="H102" s="8" t="inlineStr">
         <is>
-          <t>Justin Herbert</t>
+          <t>Jalen Hurts</t>
         </is>
       </c>
     </row>
@@ -12926,25 +12926,25 @@
       <c r="G103" s="8" t="n"/>
       <c r="H103" s="8" t="inlineStr">
         <is>
-          <t>Trevor Lawrence</t>
+          <t>Justin Herbert</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B104" s="8" t="inlineStr">
-        <is>
-          <t>Jacory Croskey-Merritt</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="B104" s="8" t="n"/>
       <c r="C104" s="8" t="n"/>
       <c r="D104" s="8" t="n"/>
       <c r="E104" s="8" t="n"/>
       <c r="F104" s="8" t="n"/>
       <c r="G104" s="8" t="n"/>
-      <c r="H104" s="8" t="n"/>
+      <c r="H104" s="8" t="inlineStr">
+        <is>
+          <t>Trevor Lawrence</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="n">
@@ -13388,29 +13388,29 @@
       </c>
       <c r="B22" s="8" t="n"/>
       <c r="C22" s="8" t="n"/>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Chris Olave</t>
-        </is>
-      </c>
+      <c r="D22" s="8" t="n"/>
       <c r="E22" s="8" t="n"/>
-      <c r="F22" s="8" t="n"/>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Trey McBride</t>
+        </is>
+      </c>
       <c r="G22" s="8" t="n"/>
       <c r="H22" s="8" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B23" s="8" t="n"/>
       <c r="C23" s="8" t="n"/>
-      <c r="D23" s="8" t="n"/>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Chris Olave</t>
+        </is>
+      </c>
       <c r="E23" s="8" t="n"/>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>Trey McBride</t>
-        </is>
-      </c>
+      <c r="F23" s="8" t="n"/>
       <c r="G23" s="8" t="n"/>
       <c r="H23" s="8" t="n"/>
     </row>
@@ -13598,7 +13598,7 @@
       <c r="C35" s="8" t="n"/>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>A.J. Brown</t>
+          <t>Mike Evans</t>
         </is>
       </c>
       <c r="E35" s="8" t="n"/>
@@ -13608,13 +13608,13 @@
     </row>
     <row r="36">
       <c r="A36" s="7" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B36" s="8" t="n"/>
       <c r="C36" s="8" t="n"/>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>Mike Evans</t>
+          <t>A.J. Brown</t>
         </is>
       </c>
       <c r="E36" s="8" t="n"/>
@@ -14014,7 +14014,7 @@
       <c r="C61" s="8" t="n"/>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>Terry McLaurin</t>
+          <t>Michael Wilson</t>
         </is>
       </c>
       <c r="E61" s="8" t="n"/>
@@ -14024,15 +14024,15 @@
     </row>
     <row r="62">
       <c r="A62" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="B62" s="8" t="n"/>
+        <v>11</v>
+      </c>
+      <c r="B62" s="8" t="inlineStr">
+        <is>
+          <t>MarShawn Lloyd</t>
+        </is>
+      </c>
       <c r="C62" s="8" t="n"/>
-      <c r="D62" s="8" t="inlineStr">
-        <is>
-          <t>Michael Wilson</t>
-        </is>
-      </c>
+      <c r="D62" s="8" t="n"/>
       <c r="E62" s="8" t="n"/>
       <c r="F62" s="8" t="n"/>
       <c r="G62" s="8" t="n"/>
@@ -14044,7 +14044,7 @@
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>MarShawn Lloyd</t>
+          <t>David Montgomery</t>
         </is>
       </c>
       <c r="C63" s="8" t="n"/>
@@ -14058,13 +14058,13 @@
       <c r="A64" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="B64" s="8" t="inlineStr">
-        <is>
-          <t>David Montgomery</t>
-        </is>
-      </c>
+      <c r="B64" s="8" t="n"/>
       <c r="C64" s="8" t="n"/>
-      <c r="D64" s="8" t="n"/>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>DJ Moore</t>
+        </is>
+      </c>
       <c r="E64" s="8" t="n"/>
       <c r="F64" s="8" t="n"/>
       <c r="G64" s="8" t="n"/>
@@ -14078,7 +14078,7 @@
       <c r="C65" s="8" t="n"/>
       <c r="D65" s="8" t="inlineStr">
         <is>
-          <t>DJ Moore</t>
+          <t>Jameson Williams</t>
         </is>
       </c>
       <c r="E65" s="8" t="n"/>
@@ -14094,7 +14094,7 @@
       <c r="C66" s="8" t="n"/>
       <c r="D66" s="8" t="inlineStr">
         <is>
-          <t>Jameson Williams</t>
+          <t>Terry McLaurin</t>
         </is>
       </c>
       <c r="E66" s="8" t="n"/>
@@ -14184,17 +14184,17 @@
     </row>
     <row r="72">
       <c r="A72" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="B72" s="8" t="inlineStr">
-        <is>
-          <t>Rachaad White</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B72" s="8" t="n"/>
       <c r="C72" s="8" t="n"/>
       <c r="D72" s="8" t="n"/>
       <c r="E72" s="8" t="n"/>
-      <c r="F72" s="8" t="n"/>
+      <c r="F72" s="8" t="inlineStr">
+        <is>
+          <t>Isaiah Likely</t>
+        </is>
+      </c>
       <c r="G72" s="8" t="n"/>
       <c r="H72" s="8" t="n"/>
     </row>
@@ -14202,15 +14202,15 @@
       <c r="A73" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B73" s="8" t="n"/>
+      <c r="B73" s="8" t="inlineStr">
+        <is>
+          <t>Rachaad White</t>
+        </is>
+      </c>
       <c r="C73" s="8" t="n"/>
       <c r="D73" s="8" t="n"/>
       <c r="E73" s="8" t="n"/>
-      <c r="F73" s="8" t="inlineStr">
-        <is>
-          <t>Isaiah Likely</t>
-        </is>
-      </c>
+      <c r="F73" s="8" t="n"/>
       <c r="G73" s="8" t="n"/>
       <c r="H73" s="8" t="n"/>
     </row>
@@ -15088,7 +15088,7 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Ashton Jeanty</t>
+          <t>Derrick Henry</t>
         </is>
       </c>
       <c r="C18" s="8" t="n"/>
@@ -15104,7 +15104,7 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Chase Brown</t>
+          <t>Ashton Jeanty</t>
         </is>
       </c>
       <c r="C19" s="8" t="n"/>
@@ -15118,31 +15118,31 @@
       <c r="A20" s="7" t="n">
         <v>44</v>
       </c>
-      <c r="B20" s="8" t="n"/>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Chase Brown</t>
+        </is>
+      </c>
       <c r="C20" s="8" t="n"/>
       <c r="D20" s="8" t="n"/>
       <c r="E20" s="8" t="n"/>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>Trey McBride</t>
-        </is>
-      </c>
+      <c r="F20" s="8" t="n"/>
       <c r="G20" s="8" t="n"/>
       <c r="H20" s="8" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
-        <v>43</v>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>Derrick Henry</t>
-        </is>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="B21" s="8" t="n"/>
       <c r="C21" s="8" t="n"/>
       <c r="D21" s="8" t="n"/>
       <c r="E21" s="8" t="n"/>
-      <c r="F21" s="8" t="n"/>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Trey McBride</t>
+        </is>
+      </c>
       <c r="G21" s="8" t="n"/>
       <c r="H21" s="8" t="n"/>
     </row>
@@ -15164,7 +15164,7 @@
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B23" s="8" t="n"/>
       <c r="C23" s="8" t="n"/>
@@ -15346,7 +15346,7 @@
       <c r="C34" s="8" t="n"/>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>A.J. Brown</t>
+          <t>Mike Evans</t>
         </is>
       </c>
       <c r="E34" s="8" t="n"/>
@@ -15362,7 +15362,7 @@
       <c r="C35" s="8" t="n"/>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>Garrett Wilson</t>
+          <t>A.J. Brown</t>
         </is>
       </c>
       <c r="E35" s="8" t="n"/>
@@ -15372,13 +15372,13 @@
     </row>
     <row r="36">
       <c r="A36" s="7" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B36" s="8" t="n"/>
       <c r="C36" s="8" t="n"/>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>Mike Evans</t>
+          <t>Garrett Wilson</t>
         </is>
       </c>
       <c r="E36" s="8" t="n"/>
@@ -15778,7 +15778,7 @@
       <c r="C61" s="8" t="n"/>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>Terry McLaurin</t>
+          <t>Michael Wilson</t>
         </is>
       </c>
       <c r="E61" s="8" t="n"/>
@@ -15788,15 +15788,15 @@
     </row>
     <row r="62">
       <c r="A62" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="B62" s="8" t="n"/>
+        <v>9</v>
+      </c>
+      <c r="B62" s="8" t="inlineStr">
+        <is>
+          <t>MarShawn Lloyd</t>
+        </is>
+      </c>
       <c r="C62" s="8" t="n"/>
-      <c r="D62" s="8" t="inlineStr">
-        <is>
-          <t>Michael Wilson</t>
-        </is>
-      </c>
+      <c r="D62" s="8" t="n"/>
       <c r="E62" s="8" t="n"/>
       <c r="F62" s="8" t="n"/>
       <c r="G62" s="8" t="n"/>
@@ -15808,7 +15808,7 @@
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>MarShawn Lloyd</t>
+          <t>David Montgomery</t>
         </is>
       </c>
       <c r="C63" s="8" t="n"/>
@@ -15822,13 +15822,13 @@
       <c r="A64" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B64" s="8" t="inlineStr">
-        <is>
-          <t>David Montgomery</t>
-        </is>
-      </c>
+      <c r="B64" s="8" t="n"/>
       <c r="C64" s="8" t="n"/>
-      <c r="D64" s="8" t="n"/>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>DJ Moore</t>
+        </is>
+      </c>
       <c r="E64" s="8" t="n"/>
       <c r="F64" s="8" t="n"/>
       <c r="G64" s="8" t="n"/>
@@ -15842,7 +15842,7 @@
       <c r="C65" s="8" t="n"/>
       <c r="D65" s="8" t="inlineStr">
         <is>
-          <t>DJ Moore</t>
+          <t>Jameson Williams</t>
         </is>
       </c>
       <c r="E65" s="8" t="n"/>
@@ -15858,7 +15858,7 @@
       <c r="C66" s="8" t="n"/>
       <c r="D66" s="8" t="inlineStr">
         <is>
-          <t>Jameson Williams</t>
+          <t>Terry McLaurin</t>
         </is>
       </c>
       <c r="E66" s="8" t="n"/>
@@ -15948,17 +15948,17 @@
     </row>
     <row r="72">
       <c r="A72" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="B72" s="8" t="inlineStr">
-        <is>
-          <t>Rachaad White</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="B72" s="8" t="n"/>
       <c r="C72" s="8" t="n"/>
       <c r="D72" s="8" t="n"/>
       <c r="E72" s="8" t="n"/>
-      <c r="F72" s="8" t="n"/>
+      <c r="F72" s="8" t="inlineStr">
+        <is>
+          <t>Isaiah Likely</t>
+        </is>
+      </c>
       <c r="G72" s="8" t="n"/>
       <c r="H72" s="8" t="n"/>
     </row>
@@ -15966,15 +15966,15 @@
       <c r="A73" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B73" s="8" t="n"/>
+      <c r="B73" s="8" t="inlineStr">
+        <is>
+          <t>Rachaad White</t>
+        </is>
+      </c>
       <c r="C73" s="8" t="n"/>
       <c r="D73" s="8" t="n"/>
       <c r="E73" s="8" t="n"/>
-      <c r="F73" s="8" t="inlineStr">
-        <is>
-          <t>Isaiah Likely</t>
-        </is>
-      </c>
+      <c r="F73" s="8" t="n"/>
       <c r="G73" s="8" t="n"/>
       <c r="H73" s="8" t="n"/>
     </row>
@@ -16190,45 +16190,45 @@
       <c r="A87" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B87" s="8" t="n"/>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>Jordan Mason</t>
+        </is>
+      </c>
       <c r="C87" s="8" t="n"/>
       <c r="D87" s="8" t="n"/>
       <c r="E87" s="8" t="n"/>
       <c r="F87" s="8" t="n"/>
       <c r="G87" s="8" t="n"/>
-      <c r="H87" s="8" t="inlineStr">
-        <is>
-          <t>Jayden Daniels</t>
-        </is>
-      </c>
+      <c r="H87" s="8" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B88" s="8" t="n"/>
+      <c r="B88" s="8" t="inlineStr">
+        <is>
+          <t>Woody Marks</t>
+        </is>
+      </c>
       <c r="C88" s="8" t="n"/>
       <c r="D88" s="8" t="n"/>
       <c r="E88" s="8" t="n"/>
       <c r="F88" s="8" t="n"/>
       <c r="G88" s="8" t="n"/>
-      <c r="H88" s="8" t="inlineStr">
-        <is>
-          <t>Dak Prescott</t>
-        </is>
-      </c>
+      <c r="H88" s="8" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B89" s="8" t="inlineStr">
-        <is>
-          <t>Jordan Mason</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="B89" s="8" t="n"/>
       <c r="C89" s="8" t="n"/>
-      <c r="D89" s="8" t="n"/>
+      <c r="D89" s="8" t="inlineStr">
+        <is>
+          <t>Brian Thomas Jr.</t>
+        </is>
+      </c>
       <c r="E89" s="8" t="n"/>
       <c r="F89" s="8" t="n"/>
       <c r="G89" s="8" t="n"/>
@@ -16236,51 +16236,51 @@
     </row>
     <row r="90">
       <c r="A90" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B90" s="8" t="inlineStr">
-        <is>
-          <t>Woody Marks</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="B90" s="8" t="n"/>
       <c r="C90" s="8" t="n"/>
       <c r="D90" s="8" t="n"/>
       <c r="E90" s="8" t="n"/>
-      <c r="F90" s="8" t="n"/>
+      <c r="F90" s="8" t="inlineStr">
+        <is>
+          <t>Tucker Kraft</t>
+        </is>
+      </c>
       <c r="G90" s="8" t="n"/>
       <c r="H90" s="8" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B91" s="8" t="inlineStr">
-        <is>
-          <t>Jonathon Brooks</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="B91" s="8" t="n"/>
       <c r="C91" s="8" t="n"/>
       <c r="D91" s="8" t="n"/>
       <c r="E91" s="8" t="n"/>
       <c r="F91" s="8" t="n"/>
       <c r="G91" s="8" t="n"/>
-      <c r="H91" s="8" t="n"/>
+      <c r="H91" s="8" t="inlineStr">
+        <is>
+          <t>Jayden Daniels</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B92" s="8" t="inlineStr">
-        <is>
-          <t>Mike Washington Jr.</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="B92" s="8" t="n"/>
       <c r="C92" s="8" t="n"/>
       <c r="D92" s="8" t="n"/>
       <c r="E92" s="8" t="n"/>
       <c r="F92" s="8" t="n"/>
       <c r="G92" s="8" t="n"/>
-      <c r="H92" s="8" t="n"/>
+      <c r="H92" s="8" t="inlineStr">
+        <is>
+          <t>Dak Prescott</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="7" t="n">
@@ -16288,7 +16288,7 @@
       </c>
       <c r="B93" s="8" t="inlineStr">
         <is>
-          <t>Rico Dowdle</t>
+          <t>Jonathon Brooks</t>
         </is>
       </c>
       <c r="C93" s="8" t="n"/>
@@ -16304,7 +16304,7 @@
       </c>
       <c r="B94" s="8" t="inlineStr">
         <is>
-          <t>J.K. Dobbins</t>
+          <t>Mike Washington Jr.</t>
         </is>
       </c>
       <c r="C94" s="8" t="n"/>
@@ -16320,7 +16320,7 @@
       </c>
       <c r="B95" s="8" t="inlineStr">
         <is>
-          <t>Blake Corum</t>
+          <t>Rico Dowdle</t>
         </is>
       </c>
       <c r="C95" s="8" t="n"/>
@@ -16336,7 +16336,7 @@
       </c>
       <c r="B96" s="8" t="inlineStr">
         <is>
-          <t>Jacory Croskey-Merritt</t>
+          <t>J.K. Dobbins</t>
         </is>
       </c>
       <c r="C96" s="8" t="n"/>
@@ -16350,13 +16350,13 @@
       <c r="A97" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B97" s="8" t="n"/>
+      <c r="B97" s="8" t="inlineStr">
+        <is>
+          <t>Blake Corum</t>
+        </is>
+      </c>
       <c r="C97" s="8" t="n"/>
-      <c r="D97" s="8" t="inlineStr">
-        <is>
-          <t>Brian Thomas Jr.</t>
-        </is>
-      </c>
+      <c r="D97" s="8" t="n"/>
       <c r="E97" s="8" t="n"/>
       <c r="F97" s="8" t="n"/>
       <c r="G97" s="8" t="n"/>
@@ -16366,13 +16366,13 @@
       <c r="A98" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B98" s="8" t="n"/>
+      <c r="B98" s="8" t="inlineStr">
+        <is>
+          <t>Jacory Croskey-Merritt</t>
+        </is>
+      </c>
       <c r="C98" s="8" t="n"/>
-      <c r="D98" s="8" t="inlineStr">
-        <is>
-          <t>Marvin Harrison Jr.</t>
-        </is>
-      </c>
+      <c r="D98" s="8" t="n"/>
       <c r="E98" s="8" t="n"/>
       <c r="F98" s="8" t="n"/>
       <c r="G98" s="8" t="n"/>
@@ -16386,7 +16386,7 @@
       <c r="C99" s="8" t="n"/>
       <c r="D99" s="8" t="inlineStr">
         <is>
-          <t>Quentin Johnston</t>
+          <t>Marvin Harrison Jr.</t>
         </is>
       </c>
       <c r="E99" s="8" t="n"/>
@@ -16402,7 +16402,7 @@
       <c r="C100" s="8" t="n"/>
       <c r="D100" s="8" t="inlineStr">
         <is>
-          <t>Chris Godwin Jr.</t>
+          <t>Quentin Johnston</t>
         </is>
       </c>
       <c r="E100" s="8" t="n"/>
@@ -16418,7 +16418,7 @@
       <c r="C101" s="8" t="n"/>
       <c r="D101" s="8" t="inlineStr">
         <is>
-          <t>Ja'Kobi Lane</t>
+          <t>Chris Godwin Jr.</t>
         </is>
       </c>
       <c r="E101" s="8" t="n"/>
@@ -16432,13 +16432,13 @@
       </c>
       <c r="B102" s="8" t="n"/>
       <c r="C102" s="8" t="n"/>
-      <c r="D102" s="8" t="n"/>
+      <c r="D102" s="8" t="inlineStr">
+        <is>
+          <t>Ja'Kobi Lane</t>
+        </is>
+      </c>
       <c r="E102" s="8" t="n"/>
-      <c r="F102" s="8" t="inlineStr">
-        <is>
-          <t>Tucker Kraft</t>
-        </is>
-      </c>
+      <c r="F102" s="8" t="n"/>
       <c r="G102" s="8" t="n"/>
       <c r="H102" s="8" t="n"/>
     </row>

</xml_diff>